<commit_message>
Version 112: home-screen icon and full-screen app mode
Adds apple-touch-icon, 192/512 icons and a web manifest to the public site.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I110"/>
+  <dimension ref="A1:I111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5408,8 +5408,55 @@
       </c>
       <c r="I110" s="2" t="inlineStr"/>
     </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>Home-screen icon for iPhone and Android: Add to Home Screen from the public site shows a Subscription Keeper icon, named Sub Keeper, and opens full screen</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>Public site</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H111" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
+          <t>Icon files and manifest in the repo root; source in app-prototype/site-icons</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I110"/>
+  <autoFilter ref="A1:I111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v113: Guess my total and Popular subscriptions on Overview
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I111"/>
+  <dimension ref="A1:I113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5455,8 +5455,102 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>New "Guess my total" card on Overview for an empty list: quick yes/no and how-many questions give a rough monthly estimate, labeled as an estimate and compared with the US adult average</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>Each answer counts the median confirmed list price of that category's default plans in the catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>New "Popular subscriptions" card on Overview: well-known services available in the user's country with one-tap Add (shown while the list has fewer than 10)</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>Our pick of well-known services, not a ranking; added ones ask for usage like any new subscription</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I111"/>
+  <autoFilter ref="A1:I113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v114: welcome screen Popular shows the 12 popular picks only
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$114</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I113"/>
+  <dimension ref="A1:I114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5549,8 +5549,55 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Welcome screen "Popular" group now shows only the same 12 popular picks as the Overview card; every other service is listed under its category</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>Welcome screen</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>Before, Popular listed the whole catalog (over 100 services in the US)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I113"/>
+  <autoFilter ref="A1:I114"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v115: welcome categories show top 6 with See all; Apple One under Music
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I114"/>
+  <dimension ref="A1:I116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5596,8 +5596,102 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>Welcome screen: each category shows its top 6 with a "See all" link (Show fewer to collapse); popular services also appear in their own category, and picking one marks it in both places</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>Welcome screen</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H115" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I115" s="3" t="inlineStr">
+        <is>
+          <t>Top = our popular picks, then national services (known logos first), then regional, then free library options; our ordering, not a sales ranking</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>Bundles category removed: Apple One, its only entry, now sits under Music with a note naming what it bundles (Apple Music, Apple TV, Apple Arcade, iCloud+)</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>Welcome screen / Explore</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>App-side change only; services.json still says bundle</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I114"/>
+  <autoFilter ref="A1:I116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v116: Let's get started card and other-category pills on Overview
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$118</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I116"/>
+  <dimension ref="A1:I118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5493,7 +5493,7 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Replaced in v116</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr">
@@ -5540,7 +5540,7 @@
       </c>
       <c r="H113" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Removed in v116</t>
         </is>
       </c>
       <c r="I113" s="3" t="inlineStr">
@@ -5690,8 +5690,98 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>"Guess my total" became "Let's get started": Yes/No per kind of service (video, music, shopping, storage, AI, gaming, fitness, news, food); Yes shows that category's top 6 with logos to tap and add (tap again to take back off), plus a link to more in Explore. Spend estimate removed. Shows until "I'm done" or 10 subscriptions</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I117" s="3" t="inlineStr">
+        <is>
+          <t>Top 6 uses the same order as the welcome screen (our picks, not sales data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Popular subscriptions card replaced by "Explore other categories": category pills that open Explore on that category, plus See everything in Explore</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I116"/>
+  <autoFilter ref="A1:I118"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v117: Let's get started lists all national options, regional behind a link
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$119</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I118"/>
+  <dimension ref="A1:I119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5728,7 +5728,7 @@
       </c>
       <c r="H117" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v117</t>
         </is>
       </c>
       <c r="I117" s="3" t="inlineStr">
@@ -5780,8 +5780,55 @@
       </c>
       <c r="I118" s="2" t="inlineStr"/>
     </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>Let's get started: Yes now lists every option in that category that isn't regional (was top 6 plus a link to Explore); "See regional providers (N)" shows ones in the user's state, when there are any</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H119" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I119" s="3" t="inlineStr">
+        <is>
+          <t>Regional = providers limited to certain states; only those serving the user's state count</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I118"/>
+  <autoFilter ref="A1:I119"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v118: Finish setting up flow; Overview hides widgets with no data
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I119"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5827,8 +5827,102 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>New "Finish setting up" card: after picking (welcome screen or "Done picking" on Let's get started), walks each new subscription one at a time with what you pay (list price filled in) and how much you use it, with a progress bar, Save and next, and Skip for now</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>Skipped ones are picked up later by the Add your usage reminder</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>Overview hides widgets with no data: summary tiles until there's a subscription, Could save until there's a saving, Value mix until something is rated, What you use most/least until usage is entered</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H121" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I121" s="3" t="inlineStr">
+        <is>
+          <t>Value mix on Shelf/elsewhere unchanged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I119"/>
+  <autoFilter ref="A1:I121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v119: Where you can save card below Use least; Value mix last on Overview
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$123</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I121"/>
+  <dimension ref="A1:I123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5921,8 +5921,98 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>"Could save / mo" tile renamed "Where you can save" and moved below What you use least as its own card</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>Same total and See how link to Savings</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>Value mix moved to the last tile on Overview; the top row now holds only You pay each month</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I123" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I121"/>
+  <autoFilter ref="A1:I123"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v120: split You pay each month into three cards
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$124</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I123"/>
+  <dimension ref="A1:I124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6011,8 +6011,55 @@
       </c>
       <c r="I123" s="3" t="inlineStr"/>
     </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>"You pay each month" split into three cards: You pay each month, You pay each year, and Subscriptions (count)</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>Phones: monthly card full width, the other two side by side</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I123"/>
+  <autoFilter ref="A1:I124"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v121: tinted yearly and count cards on Overview
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$125</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I124"/>
+  <dimension ref="A1:I125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6058,8 +6058,55 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>You pay each year and Subscriptions cards get a lighter navy background (a wash of the monthly card's color) with white text so they blend with the header band</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H125" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I125" s="3" t="inlineStr">
+        <is>
+          <t>Follows the chosen style/theme's lead color</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I124"/>
+  <autoFilter ref="A1:I125"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v122: Where you can potentially save with savings breakdown bars
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I125"/>
+  <dimension ref="A1:I126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6105,8 +6105,55 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Savings card renamed "Where you can potentially save" and given a bar chart splitting the total into Free options, Lower tiers and alternatives, and Remove duplicates</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>Each subscription counts once at its biggest saving, so the three bars add up to the total (example data: $121.92 + $109.22 + $48.61 = $279.75)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I125"/>
+  <autoFilter ref="A1:I126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v123: tap savings bars for details; See more link
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$127</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I126"/>
+  <dimension ref="A1:I127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v123</t>
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr">
@@ -6152,8 +6152,55 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>Where you can potentially save: tap a bar to see the subscriptions in that group, each with its saving and how (free option, cheaper plan or other service, or which subscription it duplicates); tap one to open it. "See how" link renamed "See more"</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G127" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H127" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I127" s="3" t="inlineStr">
+        <is>
+          <t>Free list repeats the * note that free public options are less convenient</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I126"/>
+  <autoFilter ref="A1:I127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v124: Upcoming renewals on Overview; Value mix to Shelf
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$129</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I127"/>
+  <dimension ref="A1:I129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6006,7 +6006,7 @@
       </c>
       <c r="H123" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v124</t>
         </is>
       </c>
       <c r="I123" s="3" t="inlineStr"/>
@@ -6199,8 +6199,98 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Value mix moved to the Shelf tab</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>Overview / Shelf</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>New "Upcoming renewals" card (Value mix's old spot): subscriptions renewing in the next 30 days, soonest first (5 shown, Show more); tap one for What's new (price changes and news we know of), Features on your plan, Your usage and rating, Ways to save, and Open full details</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H129" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I129" s="3" t="inlineStr">
+        <is>
+          <t>Free subscriptions left out; What's new uses catalog recent_changes and the trending list</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I127"/>
+  <autoFilter ref="A1:I129"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v125: Tell us about yourself welcome page
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$131</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I129"/>
+  <dimension ref="A1:I131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6289,8 +6289,98 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>Welcome is now two pages. Page 1 "Tell us about yourself": icon choices I am a student, single adult, married, senior, I have kids (pick several; single/married and student/senior can't both be on), then Where do you live? Page 2 is Which subscriptions do you have? with a Back button</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>Welcome screen</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>Choices saved in the profile and set the spending average group (senior, student, family, else adult)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>Privacy text now lists what you told us about yourself among what's stored in your browser</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>Claude (follows v125)</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>Terms and privacy</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G131" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H131" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I131" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I129"/>
+  <autoFilter ref="A1:I131"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v126: age range and plan-sharing choice on welcome page
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$132</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I131"/>
+  <dimension ref="A1:I132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6327,7 +6327,7 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v126</t>
         </is>
       </c>
       <c r="I130" s="2" t="inlineStr">
@@ -6379,8 +6379,55 @@
       </c>
       <c r="I131" s="3" t="inlineStr"/>
     </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>Tell us about yourself: "single adult" and "senior" tiles replaced by How old are you? (Under 25, 25 to 34, 35 to 44, 45 to 54, 55 and over; pick one) and a checkbox "I'm open to sharing plans" (family or duo plans to split the cost)</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>Welcome screen</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>Ranges made non-overlapping; 55 and over sets the senior average. Sharing choice is saved (profile.shares) but nothing uses it yet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I131"/>
+  <autoFilter ref="A1:I132"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v127: welcome wording (student/adult, My age group)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I132"/>
+  <dimension ref="A1:I133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6426,8 +6426,51 @@
         </is>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>Welcome page 1 wording: "I am a student" is now "I am a student/adult"; "How old are you?" is now "My age group"</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>Welcome screen</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H133" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I133" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I132"/>
+  <autoFilter ref="A1:I133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v128: skip to People like you overview; admin combinations table
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$133</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$135</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I133"/>
+  <dimension ref="A1:I135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6469,8 +6469,102 @@
       </c>
       <c r="I133" s="3" t="inlineStr"/>
     </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>Welcome page 2 gets "Skip, I'll add them later". Skipping opens Overview with "What people like you pay": an estimate for the usual set of subscriptions for your age group and household at list prices, the US average for comparison, one-tap add for each (with student, duo or family plan as fits), and what that age group pays for</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>Welcome screen / Overview</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>Shares by generation from Omni Calculator survey of 500 US adults (Apr 2026); age-to-generation mapping, service per kind, 50% cutoff and plan rules are our choices</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>Admin: new People like you section with the rules (age range to survey group, service shown per kind, cutoff) and a table of all 48 combinations of age range, student, married and kids with the usual set and monthly estimate; changes save per browser</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G135" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H135" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I135" s="3" t="inlineStr">
+        <is>
+          <t>admin.plk; Back to defaults resets</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I133"/>
+  <autoFilter ref="A1:I135"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v129: Did You Know? back on Overview at the bottom
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$135</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$136</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I135"/>
+  <dimension ref="A1:I136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5188,10 +5188,14 @@
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="I105" s="3" t="inlineStr"/>
+          <t>Changed later</t>
+        </is>
+      </c>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
+          <t>Did You Know? back on Overview (bottom) in v129</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -6563,8 +6567,55 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Did You Know? moved from Shelf back to Overview, at the bottom of the page</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>Overview / Shelf</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>Shows below Upcoming renewals</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I135"/>
+  <autoFilter ref="A1:I136"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v130: Netflix and Spotify usage from your own history files
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$137</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I136"/>
+  <dimension ref="A1:I137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6614,8 +6614,55 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>Netflix and Spotify: "Get your real usage" on the subscription details. People follow the steps to download their own viewing or streaming history and choose the file; the app fills in hours month by month (read in the browser, only monthly totals kept). Shown above Usage vs cost for ChatGPT and Claude too, with an "I've requested it" marker for downloads that take days</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
+        <is>
+          <t>Subscription details</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G137" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H137" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I137" s="3" t="inlineStr">
+        <is>
+          <t>Netflix Viewing activity CSV has titles and dates only, so hours are our estimate (45 min an episode, 1 h 45 a movie); Netflix full data request and Spotify extended streaming history give real time. Steps checked against Netflix, Spotify and OpenAI help pages Oct 25, 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I136"/>
+  <autoFilter ref="A1:I137"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v131: real usage card stands out, Usage page promo, clearer unrated groups
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$140</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I137"/>
+  <dimension ref="A1:I140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6652,17 +6652,154 @@
       </c>
       <c r="H137" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed later</t>
         </is>
       </c>
       <c r="I137" s="3" t="inlineStr">
         <is>
-          <t>Netflix Viewing activity CSV has titles and dates only, so hours are our estimate (45 min an episode, 1 h 45 a movie); Netflix full data request and Spotify extended streaming history give real time. Steps checked against Netflix, Spotify and OpenAI help pages Oct 25, 2026</t>
+          <t>Netflix Viewing activity CSV has titles and dates only, so hours are our estimate (45 min an episode, 1 h 45 a movie); Netflix full data request and Spotify extended streaming history give real time. Steps checked against Netflix, Spotify and OpenAI help pages Oct 25, 2026; card restyled in v131</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>131</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>"Get your real usage" card stands out on subscription details: accent border and background, a REAL USAGE label, and a filled Choose file button</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>Subscription details</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>131</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>Usage page advertises real usage: a "Stop guessing: use your real history" card above the sliders with a button for each subscription that supports it, a "Use my real usage" link under those names, and updated intro text</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>Usage</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G139" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H139" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I139" s="3" t="inlineStr">
+        <is>
+          <t>Promo hides once every supported subscription has been pulled</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>131</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>"Not rated for last month" replaced by "Not in the &lt;month&gt; rings", grouped by reason: Tell us how much you use it, Add what you pay, Too new to rate, Paused, Not rated on use, each with a one-line explanation</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>Usage</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>Feedback: people didn't know what Not rated meant</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I137"/>
+  <autoFilter ref="A1:I140"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v132: intro page for new visitors
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$141</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I140"/>
+  <dimension ref="A1:I141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6798,8 +6798,55 @@
         </is>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>New visitors first see an intro page: headline "AI, market research and you: smarter spending on subscriptions", a three-sentence description, AI / Market research / Personalization tiles, and a Next button to the welcome page</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
+        <is>
+          <t>Intro (new visitors)</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G141" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H141" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I141" s="3" t="inlineStr">
+        <is>
+          <t>Start over and Change go straight to the welcome page, skipping the intro</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I140"/>
+  <autoFilter ref="A1:I141"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v133: tighter intro with average spend and unused share
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$142</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I141"/>
+  <dimension ref="A1:I142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6836,17 +6836,64 @@
       </c>
       <c r="H141" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed later</t>
         </is>
       </c>
       <c r="I141" s="3" t="inlineStr">
         <is>
-          <t>Start over and Change go straight to the welcome page, skipping the intro</t>
+          <t>Start over and Change go straight to the welcome page, skipping the intro; text tightened in v133</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>133</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Intro page tightened to two sentences and leads with the average spend: about $90 a month on subscriptions, with nearly $1 in every $5 going to ones rarely or never used. Source line under it; tiles and text centered, three tiles side by side on phones</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>Intro (new visitors)</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>CNET survey with YouGov, May 2025: $90/mo average, $17/mo on subscriptions rarely or never used (19%, our calculation)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I141"/>
+  <autoFilter ref="A1:I142"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v134: public site reloads itself when a newer version is out
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$143</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I142"/>
+  <dimension ref="A1:I143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6892,8 +6892,55 @@
         </is>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>134</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>Public site updates itself: when the app opens or comes back on screen, it checks the site for a newer version and reloads to it, so the iPhone home-screen icon no longer shows an old saved copy</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>Whole app (public site)</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G143" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H143" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I143" s="3" t="inlineStr">
+        <is>
+          <t>Only on the GitHub Pages site; one reload try per version</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I142"/>
+  <autoFilter ref="A1:I143"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v135: Overview links are Start from the beginning and Reset to example data
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$144</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I143"/>
+  <dimension ref="A1:I144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6939,8 +6939,55 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Overview bottom links cut to two: "Start from the beginning" (opens the intro page) and "Reset to example data" (always includes a year of usage for every example subscription). "Make test usage for the past year" removed</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>Start from the beginning replaces Start over with my own list</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I143"/>
+  <autoFilter ref="A1:I144"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v136: intro shows yearly spend; AI presents options
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$145</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I144"/>
+  <dimension ref="A1:I145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6883,12 +6883,12 @@
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed later</t>
         </is>
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>CNET survey with YouGov, May 2025: $90/mo average, $17/mo on subscriptions rarely or never used (19%, our calculation)</t>
+          <t>CNET survey with YouGov, May 2025: $90/mo average, $17/mo on subscriptions rarely or never used (19%, our calculation); yearly figures and AI wording in v136</t>
         </is>
       </c>
     </row>
@@ -6986,8 +6986,55 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>Intro page: average spend shown yearly (about $1,080 a year, over $200 of it on subscriptions rarely or never used) and AI described as presenting the options that fit you, not an assistant that answers questions</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>Intro (new visitors)</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G145" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H145" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I145" s="3" t="inlineStr">
+        <is>
+          <t>CNET/YouGov May 2025: $90/mo x 12 = $1,080; $17/mo unused = about $205/yr</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I144"/>
+  <autoFilter ref="A1:I145"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v137: intro text version B
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$146</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I145"/>
+  <dimension ref="A1:I146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7024,17 +7024,60 @@
       </c>
       <c r="H145" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed later</t>
         </is>
       </c>
       <c r="I145" s="3" t="inlineStr">
         <is>
-          <t>CNET/YouGov May 2025: $90/mo x 12 = $1,080; $17/mo unused = about $205/yr</t>
-        </is>
-      </c>
+          <t>CNET/YouGov May 2025: $90/mo x 12 = $1,080; $17/mo unused = about $205/yr; text reworded in v137</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Intro text reworded (Cuong picked version B): "Paying for subscriptions you barely use? The average American spends about $1,080 a year on them, with over $200 going to ones they rarely or never use. We use AI, market research and your own usage data to present the options that give you the most for your money."</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>Intro (new visitors)</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I145"/>
+  <autoFilter ref="A1:I146"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v138: drop redundant welcome subtitle
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I146"/>
+  <dimension ref="A1:I147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7076,8 +7076,55 @@
       </c>
       <c r="I146" s="2" t="inlineStr"/>
     </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>Welcome page: removed the "Track what you pay for..." line under the heading, since the intro page now covers it</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>Welcome screen</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G147" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H147" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I147" s="3" t="inlineStr">
+        <is>
+          <t>The line also said the list stays in this browser; that is still in the Privacy page</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I146"/>
+  <autoFilter ref="A1:I147"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v139: Back link on welcome page 1
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$147</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$148</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I147"/>
+  <dimension ref="A1:I148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7123,8 +7123,55 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Welcome page 1 (Tell us about yourself) gets a "Back" link to the intro page, placed like the one on page 2</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>Welcome screen</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>Choices made on the page are kept</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I147"/>
+  <autoFilter ref="A1:I148"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v140: intro headline Smarter Spending on Subscriptions
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$149</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I148"/>
+  <dimension ref="A1:I149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6841,7 +6841,7 @@
       </c>
       <c r="I141" s="3" t="inlineStr">
         <is>
-          <t>Start over and Change go straight to the welcome page, skipping the intro; text tightened in v133</t>
+          <t>Start over and Change go straight to the welcome page, skipping the intro; text tightened in v133; headline changed in v140</t>
         </is>
       </c>
     </row>
@@ -7170,8 +7170,55 @@
         </is>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>Intro page headline changed to "Smarter Spending on Subscriptions"</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>Intro (new visitors)</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I149" s="3" t="inlineStr">
+        <is>
+          <t>Was "AI, market research and you: smarter spending on subscriptions"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I148"/>
+  <autoFilter ref="A1:I149"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v141: intro sentence about AI, market research and information you provide
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$150</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I149"/>
+  <dimension ref="A1:I150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7071,10 +7071,14 @@
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="I146" s="2" t="inlineStr"/>
+          <t>Changed later</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>last sentence reworded in v141</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -7217,8 +7221,55 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>141</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Intro text: last sentence now reads "We use AI, market research, and information you provide us to present the options that give you the most for your money."</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>Intro (new visitors)</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>Was "...and your own usage data..."</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I149"/>
+  <autoFilter ref="A1:I150"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v142: intro says information you share
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$151</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I150"/>
+  <dimension ref="A1:I151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7259,17 +7259,60 @@
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed later</t>
         </is>
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>Was "...and your own usage data..."</t>
-        </is>
-      </c>
+          <t>Was "...and your own usage data..."; reworded in v142</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>142</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>Intro text: "information you provide us" changed to "information you share"</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>Intro (new visitors)</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H151" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I151" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I150"/>
+  <autoFilter ref="A1:I151"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v143: shorter welcome hint
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$152</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I151"/>
+  <dimension ref="A1:I152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7311,8 +7311,55 @@
       </c>
       <c r="I151" s="3" t="inlineStr"/>
     </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Welcome page: text under Tell us about yourself now reads "Pick all that apply. It helps us suggest plans that fit you."</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>Welcome screen</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>Was "...plans that fit, like student, family or senior pricing."</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I151"/>
+  <autoFilter ref="A1:I152"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v144: example ChatGPT has no pause
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$153</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I152"/>
+  <dimension ref="A1:I153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7358,8 +7358,55 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>Example data: ChatGPT no longer has a pause (it was paused Sep 15 to Oct 15), since it confused testers. Example lists saved before this lose the sample pause once, with their usage history rebuilt</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>Example data</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G153" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H153" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I153" s="3" t="inlineStr">
+        <is>
+          <t>Only removes that exact sample pause on example subscriptions</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I152"/>
+  <autoFilter ref="A1:I153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v145: View as example households replaces help icon and example reset
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$153</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$155</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I153"/>
+  <dimension ref="A1:I155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6977,12 +6977,12 @@
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed later</t>
         </is>
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>Start from the beginning replaces Start over with my own list</t>
+          <t>Start from the beginning replaces Start over with my own list; Reset to example data removed in v145</t>
         </is>
       </c>
     </row>
@@ -7405,8 +7405,98 @@
         </is>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>View as: the header help icon is replaced by a people icon that switches the whole app between Me (your own list) and three example households: Jordan (student, under 25), Sam &amp; Alex (married, 40s, with kids) and Pat &amp; Lee (senior couple, 60s, no kids). Each has its own list, profile and a year of usage, a "Viewing as" bar with Switch, and its own saved copy with a Reset option</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>Header / whole app</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>Lists and amounts are our made-up examples; prices without a catalog list price (insurance, phone, internet) are made up. Help is still in the profile menu</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>Overview: "Reset to example data" link removed (examples now come from View as); "Start from the beginning" shows only for your own list</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G155" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H155" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I155" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I153"/>
+  <autoFilter ref="A1:I155"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v146: persona names and pictures
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$155</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$156</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I155"/>
+  <dimension ref="A1:I156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7443,12 +7443,12 @@
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed later</t>
         </is>
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>Lists and amounts are our made-up examples; prices without a catalog list price (insurance, phone, internet) are made up. Help is still in the profile menu</t>
+          <t>Lists and amounts are our made-up examples; prices without a catalog list price (insurance, phone, internet) are made up. Help is still in the profile menu; Names and pictures added in v146</t>
         </is>
       </c>
     </row>
@@ -7495,8 +7495,55 @@
       </c>
       <c r="I155" s="3" t="inlineStr"/>
     </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>View as: example households get full names (Jordan Rivera, Sam &amp; Alex Chen, Pat &amp; Lee Morgan) and drawn profile pictures matching their role, shown in the View as menu, the Viewing as bar and the header avatar; greetings use both names for couples</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>Header / whole app</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>Names are made up; pictures are drawn illustrations, not photos of real people</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I155"/>
+  <autoFilter ref="A1:I156"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v147: category counts in parentheses
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$156</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$157</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I156"/>
+  <dimension ref="A1:I157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7542,8 +7542,55 @@
         </is>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>Spending by Category: the number of subscriptions after each category is now in parentheses, for example "Lawn &amp; Pest Control (2)"</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G157" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H157" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I157" s="3" t="inlineStr">
+        <is>
+          <t>The count shows on mid-size screens; it is hidden on phones and wide screens to save space</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I156"/>
+  <autoFilter ref="A1:I157"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v148: Overview numbers compared with the average person
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$158</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I157"/>
+  <dimension ref="A1:I158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7589,8 +7589,55 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>148</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Overview: each of the three top numbers (each month, each year, number of subscriptions) now shows the average for the person's group (adult, family, student or senior, changeable) and how much more or less they have. Insurance, phone, internet and home services are left out of the comparison, since the surveys don't count them, and the note under the numbers says so</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I158" s="2" t="inlineStr">
+        <is>
+          <t>Spend: CNET/YouGov US adult $90 (May 2025); family 2x adult and senior 3/5 adult are our estimates; student $82 is our estimate from Omni Calculator ranges for ages 18-29 (Apr 2026). Count: adult 5 is our estimate from Omni ranges; senior 3 from Bango (Dec 2022); family 10 is our estimate (2x adult); student uses the adult figure</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I157"/>
+  <autoFilter ref="A1:I158"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v149: name and email on the welcome screen
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$159</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I158"/>
+  <dimension ref="A1:I159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7636,8 +7636,55 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>149</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>Welcome: First name and Last name fields right under "Tell us about yourself", and a "Your email address" field after "Where do you live?". The name is used in greetings and the profile menu; an email that isn't valid is flagged before moving on</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I159" s="3" t="inlineStr">
+        <is>
+          <t>All optional. In this prototype they are saved only in the browser (no account or server yet)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I158"/>
+  <autoFilter ref="A1:I159"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v150: location note on the welcome screen
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$160</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I159"/>
+  <dimension ref="A1:I160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7683,8 +7683,51 @@
         </is>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Welcome: a line under "Where do you live?" explains that we use your location to show you regional and local services</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I159"/>
+  <autoFilter ref="A1:I160"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v151: middle-align the intro page
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$161</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I160"/>
+  <dimension ref="A1:I161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7726,8 +7726,55 @@
       </c>
       <c r="I160" s="2" t="inlineStr"/>
     </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>151</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>Intro page: content is middle-aligned (centered top to bottom) in the space below the header, on phones and computers</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
+        <is>
+          <t>Intro</t>
+        </is>
+      </c>
+      <c r="F161" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G161" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H161" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I161" s="3" t="inlineStr">
+        <is>
+          <t>On short screens where it doesn't fit, it starts at the top and scrolls as before</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I160"/>
+  <autoFilter ref="A1:I161"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v152: quieter back links above page headings
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$163</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I161"/>
+  <dimension ref="A1:I163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7165,12 +7165,12 @@
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed later</t>
         </is>
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>Choices made on the page are kept</t>
+          <t>Choices made on the page are kept; Back link moved above the heading and restyled in v152</t>
         </is>
       </c>
     </row>
@@ -7773,8 +7773,94 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Back links are now small, quiet text above the page heading on every page that has one: both welcome steps, a service's Explore page, Give feedback, and Terms and privacy (the last two used to have a "Back to the app" button at the bottom)</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>Welcome / Explore / Feedback / Legal</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I162" s="2" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>Privacy (draft): "What stays on your device" now mentions your name and email, since the welcome screen asks for them; last updated date moved to October 25, 2026</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="inlineStr">
+        <is>
+          <t>Claude (follow-up to v149)</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G163" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H163" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I163" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I161"/>
+  <autoFilter ref="A1:I163"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v153: add services we don't list on the welcome screen; Erie Insurance
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I163"/>
+  <dimension ref="A1:I165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7859,8 +7859,102 @@
       </c>
       <c r="I163" s="3" t="inlineStr"/>
     </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>153</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Welcome (subscriptions step): a "Don't see yours?" box at the end of the list adds a service we don't list by name; a search with no match offers "Add it as your own". These go into Finish setting up like the others, where you enter what you pay</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I164" s="2" t="inlineStr">
+        <is>
+          <t>Hint under the heading now points to it instead of the Explore tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="3" t="inlineStr">
+        <is>
+          <t>153</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>Erie Insurance added for car and home insurance (no list price, like other insurers), shown only to people in the 12 states and DC it serves</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E165" s="3" t="inlineStr">
+        <is>
+          <t>Explore / Welcome</t>
+        </is>
+      </c>
+      <c r="F165" s="3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G165" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H165" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I165" s="3" t="inlineStr">
+        <is>
+          <t>States from Policygenius (Mar 2023) and LendingTree; Erie's own state page did not load, so the list needs confirming. Not in our service ratings yet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I163"/>
+  <autoFilter ref="A1:I165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v154: Household Services group on Overview
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$168</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I165"/>
+  <dimension ref="A1:I168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7627,12 +7627,12 @@
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed later</t>
         </is>
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>Spend: CNET/YouGov US adult $90 (May 2025); family 2x adult and senior 3/5 adult are our estimates; student $82 is our estimate from Omni Calculator ranges for ages 18-29 (Apr 2026). Count: adult 5 is our estimate from Omni ranges; senior 3 from Bango (Dec 2022); family 10 is our estimate (2x adult); student uses the adult figure</t>
+          <t>Spend: CNET/YouGov US adult $90 (May 2025); family 2x adult and senior 3/5 adult are our estimates; student $82 is our estimate from Omni Calculator ranges for ages 18-29 (Apr 2026). Count: adult 5 is our estimate from Omni ranges; senior 3 from Bango (Dec 2022); family 10 is our estimate (2x adult); student uses the adult figure | v154: "bills" renamed Household Services</t>
         </is>
       </c>
     </row>
@@ -7953,8 +7953,141 @@
         </is>
       </c>
     </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>154</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Overview: phone, internet, car and home insurance, home security, lawn and pest, home warranties, tech support and elder care are grouped as Household Services. A bar under the top numbers splits monthly spend and count into Subscriptions and Household Services, and the third tile reads "Subscriptions &amp; services" when you have both</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I166" s="2" t="inlineStr">
+        <is>
+          <t>Child Care &amp; Tutoring stays with subscriptions, since it is mostly tutoring and learning apps</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t>154</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>Spending by Category: the legend is grouped under Subscriptions and Household Services headings with a subtotal each; each group folds its smallest categories into its own Other row</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G167" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H167" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I167" s="3" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>154</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>Comparison with the average person: tiles say "$X in subscriptions" (was "without bills") and the note says averages cover subscriptions only, so household services are left out. Small-business tools now count as subscriptions in the comparison</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I168" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I165"/>
+  <autoFilter ref="A1:I168"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v155: phone and internet need checks, renewal reminders, Household Services checkup
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$168</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$172</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I168"/>
+  <dimension ref="A1:I172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8086,8 +8086,192 @@
       </c>
       <c r="I168" s="2" t="inlineStr"/>
     </row>
+    <row r="169">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>Phone and internet: a "What you use" (data per line and lines) or "What your home needs" (people at home, 4K streaming, video calls, gaming) section on the service's page works out what you need and says when your plan is well above it</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E169" s="3" t="inlineStr">
+        <is>
+          <t>Subscription page</t>
+        </is>
+      </c>
+      <c r="F169" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G169" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H169" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I169" s="3" t="inlineStr">
+        <is>
+          <t>Speed guide from the FCC's rough figures (HD 5-8 Mbps, 4K 25, video calls 6, gaming 4) per person, doubled for several devices at once; the doubling is our estimate. Data allowances come from catalog plan notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Savings for phone and internet now use what you need: a cheaper plan from your provider and a cheaper provider that covers your data or speed. Internet rivals only include providers that list your state, plus Starlink. Options under $5 a month are left out</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>Mobile rivals are priced per line times your number of lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="3" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>Household services: optional "Policy renews" or "Contract or promo renews" date on the service's page, used for a reminder</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E171" s="3" t="inlineStr">
+        <is>
+          <t>Subscription page</t>
+        </is>
+      </c>
+      <c r="F171" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G171" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H171" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I171" s="3" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>Overview: new Household Services checkup card with one line per household service and the next thing worth doing (promo ending, renews soon, a saving, check your plan, compare quotes, or looks fine). Tap a row to open the service</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>Free public options such as library hotspots stay on Savings but aren't used as the checkup headline for phone or internet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I168"/>
+  <autoFilter ref="A1:I172"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v156: Live TV & Cable and Electricity & Gas categories, state energy shopping links
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$172</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$175</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I172"/>
+  <dimension ref="A1:I175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8270,8 +8270,145 @@
         </is>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>New Live TV &amp; Cable category: YouTube TV, Hulu + Live TV, DIRECTV (streaming), Fubo, Sling TV and Philo with prices, plus Xfinity TV and Spectrum TV (priced by address, enter what you pay). Rated by hours watched, like video, and grouped with Household Services</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="inlineStr">
+        <is>
+          <t>Explore / Overview</t>
+        </is>
+      </c>
+      <c r="F173" s="3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G173" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H173" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I173" s="3" t="inlineStr">
+        <is>
+          <t>Prices from Streaming Price Tracker (Oct 2026) and cabletv.com (Oct 4, 2026), marked not confirmed on the official site; Philo from philo.com. DIRECTV and Fubo fees noted, not added to the price. Sling and Philo count as partial alternatives (no or few local channels)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>New Electricity &amp; Gas category (Electricity, Natural Gas), cost-only with no list price. The service page has "Ways to pay less": in states where homes can pick a supplier it links the state's official comparison site and warns about variable rates; elsewhere it says the utility sets the price</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>Explore / Subscription page</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>Supplier choice: TX, PA, OH, IL, MD, NY, NJ, MA, CT, NH, DC, DE, RI, ME for electricity; PA, OH, IL, MD, NY, NJ, DC, MI, GA for gas. Sites checked 2026-10-25; NJ, DE, RI and ME sites list suppliers rather than compare offers</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>Household Services checkup shows "Compare suppliers" for electricity or gas where your state allows supplier choice</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E175" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F175" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G175" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H175" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I175" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I172"/>
+  <autoFilter ref="A1:I175"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v157: Electricity & Gas shown in Explore only, not on the welcome screen
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$175</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$176</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I175"/>
+  <dimension ref="A1:I176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8355,7 +8355,7 @@
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v157</t>
         </is>
       </c>
       <c r="I174" s="2" t="inlineStr">
@@ -8407,8 +8407,51 @@
       </c>
       <c r="I175" s="3" t="inlineStr"/>
     </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>157</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>Electricity &amp; Gas no longer shows on the welcome screen; find it in Explore. Live TV &amp; Cable stays under Household Services, as Cuong confirmed</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I175"/>
+  <autoFilter ref="A1:I176"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v158: comparison note moved to the bottom of Overview
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$176</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$177</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I176"/>
+  <dimension ref="A1:I177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8450,8 +8450,51 @@
       </c>
       <c r="I176" s="2" t="inlineStr"/>
     </row>
+    <row r="177">
+      <c r="A177" s="3" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>Overview: the "Compared with the average ..." note (group picker, estimates, household services left out, sources) moved from under the top numbers to the bottom of the page</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E177" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F177" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G177" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H177" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I177" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I176"/>
+  <autoFilter ref="A1:I177"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v159: space under Household Services checkup; Admin and Shelf tabs respect their profile setting
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$177</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$179</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I177"/>
+  <dimension ref="A1:I179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8493,8 +8493,98 @@
       </c>
       <c r="I177" s="3" t="inlineStr"/>
     </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>159</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>Overview: space added below the Household Services checkup card, so it no longer touches What you use most</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I178" s="2" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>159</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>Admin and Shelf tabs now stay hidden when they are unchecked in the profile menu</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E179" s="3" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="F179" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G179" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H179" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I179" s="3" t="inlineStr">
+        <is>
+          <t>A tab style was overriding the hidden setting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I177"/>
+  <autoFilter ref="A1:I179"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v160: cleaner Overview tiles (no subscriptions-only line)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$180</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I179"/>
+  <dimension ref="A1:I180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v160</t>
         </is>
       </c>
       <c r="I168" s="2" t="inlineStr"/>
@@ -8583,8 +8583,55 @@
         </is>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>Overview: the top three tiles no longer show the "$X in subscriptions" line. The average and percentage stay; when you also have household services the average reads "Subs avg" because it compares subscriptions only</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>"Subs avg" label added by Claude so the percentage isn't read against the full total</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I179"/>
+  <autoFilter ref="A1:I180"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v161: Overview averages combine subscriptions and household services
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$180</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$181</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I180"/>
+  <dimension ref="A1:I181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8621,7 +8621,7 @@
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v161</t>
         </is>
       </c>
       <c r="I180" s="2" t="inlineStr">
@@ -8630,8 +8630,55 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" s="3" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>Overview: the average and percentage on the top three tiles now compare subscriptions and household services together. The average adds a published US household average for each household category you have (phone, internet, car insurance, home or renters insurance, electricity); services without one count at what you pay. The bottom note lists the sources</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F181" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G181" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H181" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I181" s="3" t="inlineStr">
+        <is>
+          <t>Averages: BLS Consumer Expenditure Survey 2024 (cell phone $1,359, vehicle insurance $1,993, electricity $1,833 a year), USTelecom 2026 Broadband Pricing Index ($69.33/mo, 2025 plans), NAIC 2022 via Triple-I (homeowners $1,569, renters $171 a year; likely higher now). Gas left out because the BLS figure averages in homes without gas. Count average = subscription average plus your number of household services</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I180"/>
+  <autoFilter ref="A1:I181"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v162: South Central regional providers
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$182</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I181"/>
+  <dimension ref="A1:I182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8677,8 +8677,55 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>162</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>South Central regional providers added (23 in TX, OK, AR and LA): 6 home internet, 6 newspapers, 6 gyms, 2 lawn and pest, 2 car wash clubs and 1 farm box. Shown only to users in the states each one serves</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>Explore</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>From the daily regional scan; 26 plans have no published price and show as not confirmed. Report: app-prototype/regional/south-central-report.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I181"/>
+  <autoFilter ref="A1:I182"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v163: Plains regional providers
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$182</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$183</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I182"/>
+  <dimension ref="A1:I183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8724,8 +8724,55 @@
         </is>
       </c>
     </row>
+    <row r="183">
+      <c r="A183" s="3" t="inlineStr">
+        <is>
+          <t>163</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>Plains regional providers added (23 in MN, IA, MO, KS, NE, ND and SD), shown only to users in the states each one serves</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>Explore</t>
+        </is>
+      </c>
+      <c r="F183" s="3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G183" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H183" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I183" s="3" t="inlineStr">
+        <is>
+          <t>From the regional scan of 2026-10-24. Report: app-prototype/regional/plains-report.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I182"/>
+  <autoFilter ref="A1:I183"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v164: Ask for a lower rate scripts when prices go up
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$183</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$185</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I183"/>
+  <dimension ref="A1:I185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8771,8 +8771,98 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>164</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>"Ask for a lower rate" on the service page for services that usually negotiate (internet, mobile, cable and DIRECTV, car and home insurance, home security, lawn and pest, newspapers). It appears only when the price is going up: you entered a higher price, a promo ends within 60 days, an insurance policy renews within 45 days, or the provider announced a price rise. It gives steps and a script with a Copy button, filled in with your price and a cheaper option when we have one</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>Subscription page</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>Telecom: Consumer Reports 2018 telecom survey (80% who tried got a better deal). Insurance: rates are filed with the state, so the script asks for discounts, a policy check and a quote match (MoneyGeek). No survey found for newspapers or home services</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>164</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>Household Services checkup shows "Price going up" with a nudge to ask for a lower rate, and renewal reminders now mention asking for discounts or a lower rate</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F185" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G185" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H185" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I185" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I183"/>
+  <autoFilter ref="A1:I185"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v165: example households show Ask for a lower rate
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$186</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I185"/>
+  <dimension ref="A1:I186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8861,8 +8861,55 @@
       </c>
       <c r="I185" s="3" t="inlineStr"/>
     </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>Example households show "Ask for a lower rate": the Chens' Verizon bill went up from $165 to $185 a month, and Pat &amp; Lee's GEICO car policy renews in 30 days. Saved example lists pick this up once</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>Examples</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>Example data only (made-up price rise)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I185"/>
+  <autoFilter ref="A1:I186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v166: Overview tiles name the comparison group with an asterisk
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$186</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$187</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I186"/>
+  <dimension ref="A1:I187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8908,8 +8908,55 @@
         </is>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" s="3" t="inlineStr">
+        <is>
+          <t>166</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>Overview tiles name the comparison group, e.g. "Family avg* $669", and the asterisk links to the note at the bottom of the page, which now starts with "*"</t>
+        </is>
+      </c>
+      <c r="D187" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E187" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F187" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G187" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H187" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I187" s="3" t="inlineStr">
+        <is>
+          <t>Claude recommended the short group label plus asterisk over a long label, to keep the tiles clean</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I186"/>
+  <autoFilter ref="A1:I187"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v167: Student/Adult label on Overview tiles
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$187</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$188</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I187"/>
+  <dimension ref="A1:I188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8955,8 +8955,55 @@
         </is>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>167</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>Overview tiles say "Student/Adult avg*" instead of "Student avg*"; averages of $1,000 or more drop the cents so they fit</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>The group picker in the bottom note still says "student"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I187"/>
+  <autoFilter ref="A1:I188"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v168: remove the student group and option; adults compare by age range
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$188</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$189</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I188"/>
+  <dimension ref="A1:I189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6468,7 +6468,7 @@
       </c>
       <c r="H133" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v168</t>
         </is>
       </c>
       <c r="I133" s="3" t="inlineStr"/>
@@ -6558,7 +6558,7 @@
       </c>
       <c r="H135" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v168</t>
         </is>
       </c>
       <c r="I135" s="3" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v168</t>
         </is>
       </c>
       <c r="I188" s="2" t="inlineStr">
@@ -9002,8 +9002,55 @@
         </is>
       </c>
     </row>
+    <row r="189">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>168</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>"Student" removed everywhere: the welcome screen no longer has a student option, the comparison groups are Adult, Family and Senior, and suggestions use the age range (under 25 and so on) plus married and kids. People-like-you no longer picks student plans. The example "Student, under 25" is now "Young adult, under 25". Saved student profiles switch to Adult</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="inlineStr">
+        <is>
+          <t>Welcome / Overview / Admin</t>
+        </is>
+      </c>
+      <c r="F189" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G189" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H189" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I189" s="3" t="inlineStr">
+        <is>
+          <t>The $82 student spending estimate is no longer used; under-25s still get the Gen Z usual set from the Omni Calculator survey</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I188"/>
+  <autoFilter ref="A1:I189"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v169: Adult tile on the welcome screen
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$189</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$190</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I189"/>
+  <dimension ref="A1:I190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9049,8 +9049,51 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>169</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>Welcome screen: "I am an adult" tile added back beside "I am married" and "I have kids". It keeps the Adult comparison group; married or kids still mean Family</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I189"/>
+  <autoFilter ref="A1:I190"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v170: intro page covers household services; tiles moved to Shelf
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$190</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$191</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I190"/>
+  <dimension ref="A1:I191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9092,8 +9092,51 @@
       </c>
       <c r="I190" s="2" t="inlineStr"/>
     </row>
+    <row r="191">
+      <c r="A191" s="3" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>Intro page: header now reads "Smarter Spending on Subscriptions &amp; Household Services", the first paragraph starts "Paying for subscriptions and services you barely use?", and the source line moved below the Next button. The three tiles (AI, Market research, Personalization) moved to the Shelf tab as "How we help"</t>
+        </is>
+      </c>
+      <c r="D191" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E191" s="3" t="inlineStr">
+        <is>
+          <t>Intro / Shelf</t>
+        </is>
+      </c>
+      <c r="F191" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G191" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H191" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I191" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I190"/>
+  <autoFilter ref="A1:I191"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 171: intro page header cleanup and larger green title
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$192</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I191"/>
+  <dimension ref="A1:I192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9135,8 +9135,51 @@
       </c>
       <c r="I191" s="3" t="inlineStr"/>
     </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>171</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>Intro page only: search, View as and profile buttons hidden; app title enlarged to fit the phone width in green; other text enlarged proportionately</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>Intro page</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I192" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I191"/>
+  <autoFilter ref="A1:I192"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 172: shorten intro source line
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$192</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$193</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I192"/>
+  <dimension ref="A1:I193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9178,8 +9178,51 @@
       </c>
       <c r="I192" s="2" t="inlineStr"/>
     </row>
+    <row r="193">
+      <c r="A193" s="3" t="inlineStr">
+        <is>
+          <t>172</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>Intro page source line shortened: the "(about $90 a month, $17 of it unused)" note removed</t>
+        </is>
+      </c>
+      <c r="D193" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E193" s="3" t="inlineStr">
+        <is>
+          <t>Intro page</t>
+        </is>
+      </c>
+      <c r="F193" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G193" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H193" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I193" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I192"/>
+  <autoFilter ref="A1:I193"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 173: about-you page header, gold welcome title, numbered subheaders
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$194</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I193"/>
+  <dimension ref="A1:I194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9176,7 +9176,11 @@
           <t>Current</t>
         </is>
       </c>
-      <c r="I192" s="2" t="inlineStr"/>
+      <c r="I192" s="2" t="inlineStr">
+        <is>
+          <t>Extended to the About you page in v173</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
@@ -9221,8 +9225,51 @@
       </c>
       <c r="I193" s="3" t="inlineStr"/>
     </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>173</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>About you page (welcome step 1): search, View as and profile buttons hidden and big green title, as on the intro page; heading changed from "Welcome to Subscription Keeper" to "We’re Glad You’re Here!" in gold, one size larger; subheaders numbered 1 to 4</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>About you page</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I194" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I193"/>
+  <autoFilter ref="A1:I194"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 174: centered Next button on about-you page
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$194</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$195</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I194"/>
+  <dimension ref="A1:I195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9268,8 +9268,51 @@
       </c>
       <c r="I194" s="2" t="inlineStr"/>
     </row>
+    <row r="195">
+      <c r="A195" s="3" t="inlineStr">
+        <is>
+          <t>174</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>About you page: "Next: your subscriptions" button renamed "Next", centered, same size as the intro page button</t>
+        </is>
+      </c>
+      <c r="D195" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E195" s="3" t="inlineStr">
+        <is>
+          <t>About you page</t>
+        </is>
+      </c>
+      <c r="F195" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G195" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H195" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I195" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I194"/>
+  <autoFilter ref="A1:I195"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 175: Back and Next buttons side by side on about-you page
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$195</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$196</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I195"/>
+  <dimension ref="A1:I196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9306,13 +9306,56 @@
       </c>
       <c r="H195" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v175</t>
         </is>
       </c>
       <c r="I195" s="3" t="inlineStr"/>
     </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>About you page: the Back link under the heading replaced by a Back button to the left of Next; both buttons natural width; "Just looking? Try it with example data" and "Keep my current list" removed from this page (still on the subscriptions page)</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>About you page</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I196" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I195"/>
+  <autoFilter ref="A1:I196"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 176: remove location and storage notes on about-you page
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$196</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$197</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I196"/>
+  <dimension ref="A1:I197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9354,8 +9354,51 @@
       </c>
       <c r="I196" s="2" t="inlineStr"/>
     </row>
+    <row r="197">
+      <c r="A197" s="3" t="inlineStr">
+        <is>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>About you page: notes "We use your location to show you regional and local services." and "In this prototype it's saved only in this browser." removed (the email error message still shows when needed)</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E197" s="3" t="inlineStr">
+        <is>
+          <t>About you page</t>
+        </is>
+      </c>
+      <c r="F197" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G197" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H197" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I197" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I196"/>
+  <autoFilter ref="A1:I197"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 177: square age group tiles on about-you page
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$197</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$198</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I197"/>
+  <dimension ref="A1:I198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9397,8 +9397,51 @@
       </c>
       <c r="I197" s="3" t="inlineStr"/>
     </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>177</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>About you page: age group options are now square tiles (3 per row) matching the section 1 tiles, each showing the range and "years old"</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>About you page</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I198" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I197"/>
+  <autoFilter ref="A1:I198"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 178: subscriptions welcome page redesign with category pills
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$198</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$199</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I198"/>
+  <dimension ref="A1:I199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9440,8 +9440,55 @@
       </c>
       <c r="I198" s="2" t="inlineStr"/>
     </row>
+    <row r="199">
+      <c r="A199" s="3" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>Subscriptions page (welcome step 2): search, View as and profile buttons hidden and big green title like the first two pages; "Welcome to Subscription Keeper" removed; sections numbered (1. Which subscriptions do you have?, 2. Want to add more?, 3. Don't see yours?); categories now under section 2 with Explore-style pills that show only the picked categories (All clears); Back link became a Back button left of Start at the bottom; "Skip, I'll add them later" and "Just looking? Try it with example data" are their own buttons; Terms of Use line and "Keep my current list" removed</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E199" s="3" t="inlineStr">
+        <is>
+          <t>Subscriptions page (welcome)</t>
+        </is>
+      </c>
+      <c r="F199" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G199" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H199" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I199" s="3" t="inlineStr">
+        <is>
+          <t>Terms of Use and Privacy are still linked from the profile menu and Help page</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I198"/>
+  <autoFilter ref="A1:I199"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 179: category dropdown on subscriptions welcome page
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$200</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I199"/>
+  <dimension ref="A1:I200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H199" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v179</t>
         </is>
       </c>
       <c r="I199" s="3" t="inlineStr">
@@ -9487,8 +9487,55 @@
         </is>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>179</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>Subscriptions page: category pills replaced by a "Pick a category" dropdown that shows one category's subscriptions at a time (AI Assistants by default, "All categories" at the end); the Start button now reads "Subscriptions Selected: X"</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>Subscriptions page (welcome)</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="inlineStr">
+        <is>
+          <t>Search still looks across every category</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I199"/>
+  <autoFilter ref="A1:I200"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 180: tinted Finish setting up card with centered buttons
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I200"/>
+  <dimension ref="A1:I201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9534,8 +9534,51 @@
         </is>
       </c>
     </row>
+    <row r="201">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>Overview: "Finish setting up" card gets a light accent-colored background and border so it stands out; its Save and Skip buttons are centered</t>
+        </is>
+      </c>
+      <c r="D201" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E201" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F201" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G201" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H201" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I201" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I200"/>
+  <autoFilter ref="A1:I201"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 181: live value rating while sliding on Usage tab
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$202</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I201"/>
+  <dimension ref="A1:I202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9577,8 +9577,55 @@
       </c>
       <c r="I201" s="3" t="inlineStr"/>
     </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>Usage tab: the Great / Fair / Costly rating next to each slider now changes live while the slider moves (was only after letting go); the value is still saved on release</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>Usage</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr">
+        <is>
+          <t>Services without a typical cost-per-use range (e.g. LA Fitness, Tinder, Adobe, DoorDash, Costco) stay Fair at any level</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I201"/>
+  <autoFilter ref="A1:I202"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 182: app renamed to MoSuBi with the bundle logo and new home-screen icon
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$202</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$204</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I202"/>
+  <dimension ref="A1:I204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5450,7 +5450,7 @@
       </c>
       <c r="H111" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Icon and name changed in v182</t>
         </is>
       </c>
       <c r="I111" s="3" t="inlineStr">
@@ -9624,8 +9624,102 @@
         </is>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" s="3" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>App renamed from Subscription Keeper to MoSuBi (Manage Subscriptions and Bills), with the new "bundle" logo (white block with a band in the app-name green #4ade80) next to the name in the header and on the opening screen</t>
+        </is>
+      </c>
+      <c r="D203" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="inlineStr">
+        <is>
+          <t>Whole app (name, header, opening screen, Terms, Sam)</t>
+        </is>
+      </c>
+      <c r="F203" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G203" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H203" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I203" s="3" t="inlineStr">
+        <is>
+          <t>Logo files in branding/mosubi; repo name and public site address unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>New home-screen and browser icon (the bundle logo); home-screen name is now MoSuBi (was Sub Keeper)</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>Home-screen app / site icons</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="inlineStr">
+        <is>
+          <t>iPhones that already added the old icon may need to remove and re-add it to see the new one</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I202"/>
+  <autoFilter ref="A1:I204"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 183: larger header logo and name; logo left-aligned on welcome pages
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$206</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I204"/>
+  <dimension ref="A1:I206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9718,8 +9718,94 @@
         </is>
       </c>
     </row>
+    <row r="205">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>Header logo and MoSuBi name are larger (24 px, was 17 px) on the main app screens</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="inlineStr">
+        <is>
+          <t>Header (all screens)</t>
+        </is>
+      </c>
+      <c r="F205" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G205" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H205" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I205" s="3" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>On the intro, About you and subscriptions welcome pages, the logo and green MoSuBi name sit on the left instead of centered</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>Welcome pages</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I206" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I204"/>
+  <autoFilter ref="A1:I206"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 184: selected-count card after section 3 and separate Next button on the subscriptions welcome page
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$206</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$207</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I206"/>
+  <dimension ref="A1:I207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9525,7 +9525,7 @@
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Button changed in v184</t>
         </is>
       </c>
       <c r="I200" s="2" t="inlineStr">
@@ -9804,8 +9804,55 @@
       </c>
       <c r="I206" s="2" t="inlineStr"/>
     </row>
+    <row r="207">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>Subscriptions welcome page: the selected count is now its own card after section 3 ("3 Subscriptions Selected"), and the bottom bar has Back and a separate Next button (was Back and a "Subscriptions Selected: X" button)</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="inlineStr">
+        <is>
+          <t>Subscriptions page (welcome)</t>
+        </is>
+      </c>
+      <c r="F207" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G207" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H207" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I207" s="3" t="inlineStr">
+        <is>
+          <t>Next does what the old count button did</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I206"/>
+  <autoFilter ref="A1:I207"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 185: name boxes on About you page are white with larger blue text
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$207</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$208</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I207"/>
+  <dimension ref="A1:I208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9851,8 +9851,55 @@
         </is>
       </c>
     </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>185</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>About you page: First name and Last name boxes have a white background and blue text at double size (26 px, was 13 px)</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>About you page (welcome)</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I208" s="2" t="inlineStr">
+        <is>
+          <t>Other boxes on the page (such as email) unchanged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I207"/>
+  <autoFilter ref="A1:I208"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 186: welcome-page boxes styled like the name boxes; selected counter above section 2
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$210</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I208"/>
+  <dimension ref="A1:I210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9898,8 +9898,98 @@
         </is>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>About you page: Country, State and Email boxes match the name boxes (white background, blue text at 26 px); Country and State now each take a full row so the larger text fits</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="inlineStr">
+        <is>
+          <t>About you page (welcome)</t>
+        </is>
+      </c>
+      <c r="F209" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G209" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H209" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I209" s="3" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>Subscriptions welcome page: the "Subscriptions Selected" counter card moves above section 2 and keeps updating as more are picked or added; the "Don't see yours?" box gets the same white background and 26 px blue text (placeholder shortened to "e.g. Hometown Gym")</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>Subscriptions page (welcome)</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I210" s="2" t="inlineStr">
+        <is>
+          <t>Counter was after section 3 in v184</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I208"/>
+  <autoFilter ref="A1:I210"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 187: remove leftover Let's get started and Explore other categories cards from Overview
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$210</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$211</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I210"/>
+  <dimension ref="A1:I211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5732,7 +5732,7 @@
       </c>
       <c r="H117" s="3" t="inlineStr">
         <is>
-          <t>Changed in v117</t>
+          <t>Removed in v187</t>
         </is>
       </c>
       <c r="I117" s="3" t="inlineStr">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Removed in v187</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr"/>
@@ -5822,7 +5822,7 @@
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Removed in v187</t>
         </is>
       </c>
       <c r="I119" s="3" t="inlineStr">
@@ -9988,8 +9988,55 @@
         </is>
       </c>
     </row>
+    <row r="211">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>Overview: removed the leftover "Let's get started" and "Explore other categories" cards. "Finish setting up" now shows whenever there are new subscriptions to set up, and "What people like you pay" (after Skip on the welcome page) stays until 10 subscriptions</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F211" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G211" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H211" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I211" s="3" t="inlineStr">
+        <is>
+          <t>Checked: nothing picked, some picked, Skip then tap a suggestion, example data; no errors. With an empty list, adding is through search or Explore</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I210"/>
+  <autoFilter ref="A1:I211"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 188: shorter subscription picker with category pills and a pinned Your list bar
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$211</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$212</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I211"/>
+  <dimension ref="A1:I212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9525,7 +9525,7 @@
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
-          <t>Button changed in v184</t>
+          <t>Replaced in v188</t>
         </is>
       </c>
       <c r="I200" s="2" t="inlineStr">
@@ -9842,7 +9842,7 @@
       </c>
       <c r="H207" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Replaced in v188</t>
         </is>
       </c>
       <c r="I207" s="3" t="inlineStr">
@@ -9979,7 +9979,7 @@
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Replaced in v188</t>
         </is>
       </c>
       <c r="I210" s="2" t="inlineStr">
@@ -10035,8 +10035,55 @@
         </is>
       </c>
     </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>Subscriptions welcome page reorganized to be short: search on top (no match offers "Add ... as your own", replacing the "Don't see yours?" section), Popular picks, then category pills with one category open at a time (12 common ones first, "More categories" for the rest, a count on pills you've picked from), and a "Your list" bar pinned to the bottom with the picked names as removable chips (first 3, "+N more") plus Back and Next</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>Subscriptions page (welcome)</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H212" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I212" s="2" t="inlineStr">
+        <is>
+          <t>Replaces the category dropdown (v179) and the counter card (v184/v186); search box gets the white, large blue style</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I211"/>
+  <autoFilter ref="A1:I212"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 189: Household Services checkup moved from Overview to the Shelf tab
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$213</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I212"/>
+  <dimension ref="A1:I213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8261,7 +8261,7 @@
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Moved to Shelf in v189</t>
         </is>
       </c>
       <c r="I172" s="2" t="inlineStr">
@@ -10082,8 +10082,55 @@
         </is>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" s="3" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>Household Services checkup card moved from Overview to the Shelf tab (still works there; tap a row to open that service)</t>
+        </is>
+      </c>
+      <c r="D213" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="inlineStr">
+        <is>
+          <t>Overview / Shelf</t>
+        </is>
+      </c>
+      <c r="F213" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G213" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H213" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I213" s="3" t="inlineStr">
+        <is>
+          <t>Shelf tab shows only when "Show the Shelf tab" is on in the profile menu</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I212"/>
+  <autoFilter ref="A1:I213"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 190: welcome setup screen asks plan and one usage question per subscription
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$213</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$214</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I213"/>
+  <dimension ref="A1:I214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10129,8 +10129,55 @@
         </is>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>New welcome screen after picking subscriptions: "Finish setting up" goes through them one at a time with two questions: 1. Which plan do you have? (plans with prices; services we don't list ask what you pay) and 2. one usage question for the value chart (e.g. hours watched a week, days used a month). Next saves and moves to the next one (Done after the last); Finish later goes to Overview, where the Finish setting up card has the rest</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>Welcome setup screen (new)</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I214" s="2" t="inlineStr">
+        <is>
+          <t>Usage left at 0 stays "not entered" so no rating is shown until they add it; cost-only services (insurance, phone, internet) skip question 2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I213"/>
+  <autoFilter ref="A1:I214"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 191: persona picker titled Demo Data - View As
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$214</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$215</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I214"/>
+  <dimension ref="A1:I215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10176,8 +10176,51 @@
         </is>
       </c>
     </row>
+    <row r="215">
+      <c r="A215" s="3" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>Persona picker title renamed from "View as" to "Demo Data - View As" (also the header button's tooltip)</t>
+        </is>
+      </c>
+      <c r="D215" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E215" s="3" t="inlineStr">
+        <is>
+          <t>View as (personas)</t>
+        </is>
+      </c>
+      <c r="F215" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G215" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H215" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I215" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I214"/>
+  <autoFilter ref="A1:I215"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 192: Add subscriptions and Manage my list on Overview
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$215</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$216</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I215"/>
+  <dimension ref="A1:I216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10219,8 +10219,55 @@
       </c>
       <c r="I215" s="3" t="inlineStr"/>
     </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>192</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>Overview: "+ Add subscriptions" and "Manage my list" buttons above Did You Know? (Add at the top under the greeting when the list is empty). Add opens the same picker as the welcome page, with ones already on your list faded; new picks are added to the list (not replacing it) and go through the Finish setting up screen. Manage my list shows every subscription with Remove, which asks to confirm</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>Overview / Manage my list (new)</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I216" s="2" t="inlineStr">
+        <is>
+          <t>Remove is also still on each subscription's own page</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I215"/>
+  <autoFilter ref="A1:I216"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 193: welcome picks are kept across Back/Next and reloads; Clear selections with confirm
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$216</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$217</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I216"/>
+  <dimension ref="A1:I217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10266,8 +10266,55 @@
         </is>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" s="3" t="inlineStr">
+        <is>
+          <t>193</t>
+        </is>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>Subscriptions welcome page keeps your picks (including ones you added yourself) when you go Back and Next or reload the page, and reopens on that page if you left with picks; new "Clear selections" link in the Your list bar asks "Clear all N selections?" before clearing</t>
+        </is>
+      </c>
+      <c r="D217" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E217" s="3" t="inlineStr">
+        <is>
+          <t>Subscriptions page (welcome)</t>
+        </is>
+      </c>
+      <c r="F217" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G217" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H217" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I217" s="3" t="inlineStr">
+        <is>
+          <t>Picks are saved in this browser only, like the rest of the list</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I216"/>
+  <autoFilter ref="A1:I217"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 194: Did You Know moved from Overview to the top of Explore
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$217</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$218</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I217"/>
+  <dimension ref="A1:I218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10313,8 +10313,51 @@
         </is>
       </c>
     </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>194</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>Did You Know? card moved from the bottom of Overview to the top of Explore (still rotates, with arrows, dots and swipe)</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>Overview / Explore</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I218" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I217"/>
+  <autoFilter ref="A1:I218"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 195: Add subscriptions and Manage my list buttons centered
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$218</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$219</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I218"/>
+  <dimension ref="A1:I219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10356,8 +10356,51 @@
       </c>
       <c r="I218" s="2" t="inlineStr"/>
     </row>
+    <row r="219">
+      <c r="A219" s="3" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>"+ Add subscriptions" and "Manage my list" buttons are centered (Overview and Manage my list page)</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>Overview / Manage my list</t>
+        </is>
+      </c>
+      <c r="F219" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I219" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I218"/>
+  <autoFilter ref="A1:I219"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 196: Go to Welcome Screen / Reset My Selections links, Back button on Manage my list
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$219</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$221</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I219"/>
+  <dimension ref="A1:I221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10399,8 +10399,94 @@
       </c>
       <c r="I219" s="3" t="inlineStr"/>
     </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t>Overview: "Start from the beginning" replaced by "Go to Welcome Screen" (keeps all data; picker shows current list ticked, only new picks are added and set up) and "Reset My Selections" (clears the list after a confirm)</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>Overview / Welcome</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="3" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>Manage My List: added a Back button beside + Add subscriptions</t>
+        </is>
+      </c>
+      <c r="D221" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="inlineStr">
+        <is>
+          <t>Manage my list</t>
+        </is>
+      </c>
+      <c r="F221" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G221" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H221" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I221" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I219"/>
+  <autoFilter ref="A1:I221"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 197: usage slider tops lowered per type of subscription
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$221</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$222</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I221"/>
+  <dimension ref="A1:I222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10485,8 +10485,55 @@
       </c>
       <c r="I221" s="3" t="inlineStr"/>
     </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>Usage slider tops lowered per type of subscription (was 100+ for most): video and music 40 hrs/wk, live TV 60, gaming 40, learning 20, AI 50 prompts/day, news 30 articles/wk, shopping and food 30 orders/mo, Prime orders under $35 20/mo, Uber One 40 trips, Evernote 60 notes, Cloaked 50 removals, CNBC 20 hrs or 30 Pro articles/wk. Top still means that much or more.</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t>Usage / Setup</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I222" s="2" t="inlineStr">
+        <is>
+          <t>From tester feedback that 100+ was overkill</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I221"/>
+  <autoFilter ref="A1:I222"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 198: light borders on cards, more space between Overview widgets
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$222</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$223</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I222"/>
+  <dimension ref="A1:I223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10532,8 +10532,55 @@
         </is>
       </c>
     </row>
+    <row r="223">
+      <c r="A223" s="3" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>White cards get a light border across the app; on Overview, more space between widgets and a thin line under each widget title</t>
+        </is>
+      </c>
+      <c r="D223" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>Overview / all pages</t>
+        </is>
+      </c>
+      <c r="F223" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G223" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H223" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I223" s="3" t="inlineStr">
+        <is>
+          <t>From tester feedback that Overview was still busy</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I222"/>
+  <autoFilter ref="A1:I223"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 199: Overview footnotes behind an i circle icon
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$223</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$224</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I223"/>
+  <dimension ref="A1:I224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10579,8 +10579,51 @@
         </is>
       </c>
     </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>199</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>Footnotes behind an "i" circle icon (reusable on any screen): Overview's averages and sources note opens from an i on "You pay each month" (the * after "avg" is gone), and the ranking note from an i next to "What you use most"</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I224" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I223"/>
+  <autoFilter ref="A1:I224"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 200: remove top Back to Overview link on Manage my list
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$224</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$225</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I224"/>
+  <dimension ref="A1:I225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10622,8 +10622,51 @@
       </c>
       <c r="I224" s="2" t="inlineStr"/>
     </row>
+    <row r="225">
+      <c r="A225" s="3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>Manage my list: removed the top "Back to Overview" link (the Back button at the bottom stays)</t>
+        </is>
+      </c>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>Manage my list</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G225" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H225" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I225" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I224"/>
+  <autoFilter ref="A1:I225"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 201: Welcome Screen and Reset My Selections links centered
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$225</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$226</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I225"/>
+  <dimension ref="A1:I226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10665,8 +10665,51 @@
       </c>
       <c r="I225" s="3" t="inlineStr"/>
     </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>Overview: "Go to Welcome Screen" renamed "Welcome Screen"; it and "Reset My Selections" are centered</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I226" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I225"/>
+  <autoFilter ref="A1:I226"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 202: Add subscriptions basket counts what's already on the list
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$226</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$227</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I226"/>
+  <dimension ref="A1:I227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10708,8 +10708,51 @@
       </c>
       <c r="I226" s="2" t="inlineStr"/>
     </row>
+    <row r="227">
+      <c r="A227" s="3" t="inlineStr">
+        <is>
+          <t>202</t>
+        </is>
+      </c>
+      <c r="B227" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>Fix: "+ Add subscriptions" picker's Your list counted only new picks (showed 0). It now counts and shows what's already on your list (faded, no x) plus new picks</t>
+        </is>
+      </c>
+      <c r="D227" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E227" s="3" t="inlineStr">
+        <is>
+          <t>Add subscriptions</t>
+        </is>
+      </c>
+      <c r="F227" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G227" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H227" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I227" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I226"/>
+  <autoFilter ref="A1:I227"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 203: yearly and count tile averages moved into the i panel
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$227</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$228</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I227"/>
+  <dimension ref="A1:I228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10751,8 +10751,51 @@
       </c>
       <c r="I227" s="3" t="inlineStr"/>
     </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>203</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>Overview: "You pay each year" and "Subscriptions &amp; services" tiles show just their number; their average and % moved into the i panel (opened from You pay each month)</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I228" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I227"/>
+  <autoFilter ref="A1:I228"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 204: fix setup wording for services rated on doing their job
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$228</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$229</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I228"/>
+  <dimension ref="A1:I229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10794,8 +10794,51 @@
       </c>
       <c r="I228" s="2" t="inlineStr"/>
     </row>
+    <row r="229">
+      <c r="A229" s="3" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>Fix: setup question for 1Password and other services rated on "doing its job" (antivirus, internet, phone, cameras, pest/lawn...) said you'd tick off what you used. It's now "How we rate it" and explains you tick anything that went wrong (e.g. sync, autofill or login problems); nothing ticked means it's working</t>
+        </is>
+      </c>
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E229" s="3" t="inlineStr">
+        <is>
+          <t>Setup / Overview</t>
+        </is>
+      </c>
+      <c r="F229" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I229" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I228"/>
+  <autoFilter ref="A1:I229"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 205: Everything's going great box on monthly problem checks
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JakwMhYzgScL99LoRY7oLY
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$229</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$230</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I229"/>
+  <dimension ref="A1:I230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10837,8 +10837,51 @@
       </c>
       <c r="I229" s="3" t="inlineStr"/>
     </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>205</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>"Everything's going great!" box added to the monthly "Anything go wrong?" checks for services rated on doing their job (1Password, antivirus, internet, phone, cameras, pest/lawn...). It and the problem boxes clear each other; it never counts as a problem</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
+          <t>Usage / Subscription sheet</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H230" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I230" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I229"/>
+  <autoFilter ref="A1:I230"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 206: hide household split bar until a household service has a price
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$230</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$231</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I230"/>
+  <dimension ref="A1:I231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10880,8 +10880,51 @@
       </c>
       <c r="I230" s="2" t="inlineStr"/>
     </row>
+    <row r="231">
+      <c r="A231" s="3" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>Overview: the Subscriptions vs Household Services bar under the tiles is hidden until at least one household service has a price (insurers like Progressive have no list price, so they showed as $0.00); the legend notes household services still without a price; version label corrected (showed 196)</t>
+        </is>
+      </c>
+      <c r="D231" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E231" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F231" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G231" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H231" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I231" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I230"/>
+  <autoFilter ref="A1:I231"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 207: Welcome Back page and fix for services with no published price
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$231</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$233</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I231"/>
+  <dimension ref="A1:I233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10923,8 +10923,98 @@
       </c>
       <c r="I231" s="3" t="inlineStr"/>
     </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>207</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>New "Welcome Back" page for returning visitors (once per visit): walks through missing info one item at a time (a subscription's price or usage, then name, age group, state) with Save and next, Skip and "Come back later"; when nothing is missing but a subscription is rated Costly, it offers to review cheaper options</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="inlineStr">
+        <is>
+          <t>Welcome Back (new)</t>
+        </is>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G232" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H232" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I232" s="2" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="3" t="inlineStr">
+        <is>
+          <t>207</t>
+        </is>
+      </c>
+      <c r="B233" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C233" s="3" t="inlineStr">
+        <is>
+          <t>Fix: services with no published price (Progressive and other insurers, some regional providers) were counted as $0. They now ask what you pay, in Finish setting up and on Welcome Back, and existing ones at $0 are asked again</t>
+        </is>
+      </c>
+      <c r="D233" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E233" s="3" t="inlineStr">
+        <is>
+          <t>Finish setting up / prices</t>
+        </is>
+      </c>
+      <c r="F233" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G233" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H233" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I233" s="3" t="inlineStr">
+        <is>
+          <t>Cause: a missing yearly price was computed as $0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I231"/>
+  <autoFilter ref="A1:I233"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 208: Welcome Back intro text with gold lead sentence
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$233</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$234</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I233"/>
+  <dimension ref="A1:I234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11013,8 +11013,51 @@
         </is>
       </c>
     </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>208</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>Welcome Back: intro text changed to "We noticed some information is missing. Completing this makes your ratings and savings more accurate."; the first sentence is larger and gold</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="inlineStr">
+        <is>
+          <t>Welcome Back</t>
+        </is>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G234" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H234" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I234" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I233"/>
+  <autoFilter ref="A1:I234"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 209: add Mountain regional providers
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$234</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$235</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I234"/>
+  <dimension ref="A1:I235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11056,8 +11056,55 @@
       </c>
       <c r="I234" s="2" t="inlineStr"/>
     </row>
+    <row r="235">
+      <c r="A235" s="3" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="B235" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="inlineStr">
+        <is>
+          <t>Regional providers: Mountain region added (CO, UT, WY, MT, ID, NV): 21 providers (6 internet, 6 news, 4 fitness, 2 car wash, Rocky Mountain Power Blue Sky, Union Wireless, a farm box), shown only to people in the states they serve</t>
+        </is>
+      </c>
+      <c r="D235" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E235" s="3" t="inlineStr">
+        <is>
+          <t>Explore / regional</t>
+        </is>
+      </c>
+      <c r="F235" s="3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G235" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H235" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I235" s="3" t="inlineStr">
+        <is>
+          <t>174 regional providers in total; 9 plans not confirmed, 18 with no published price</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I234"/>
+  <autoFilter ref="A1:I235"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v210: Finish setting up picks payment and usage frequency; restyled card
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$235</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$236</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I235"/>
+  <dimension ref="A1:I236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9572,7 +9572,7 @@
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v210</t>
         </is>
       </c>
       <c r="I201" s="3" t="inlineStr"/>
@@ -11103,8 +11103,55 @@
         </is>
       </c>
     </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>Finish setting up (Overview card and setup page): pick how often you pay (a month, every 3 months, every 6 months, a year) and how usage is counted (a day, a week, a month, a year, where it fits the measure); card restyled to match the welcome screens (page background, white question cards, larger text)</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr">
+        <is>
+          <t>Finish setting up</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G236" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H236" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I236" s="2" t="inlineStr">
+        <is>
+          <t>Prices paid every 3 or 6 months are stored as a monthly amount</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I235"/>
+  <autoFilter ref="A1:I236"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v211: Password managers track logins filled a day and are rated on use
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$236</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$237</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I236"/>
+  <dimension ref="A1:I237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v211 (password managers)</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
@@ -11150,8 +11150,55 @@
         </is>
       </c>
     </row>
+    <row r="237">
+      <c r="A237" s="3" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>Password managers (1Password and others) now track usage: "Logins filled a day" slider, rated Great value or Costly per login instead of on doing its job</t>
+        </is>
+      </c>
+      <c r="D237" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E237" s="3" t="inlineStr">
+        <is>
+          <t>Usage / Value rating</t>
+        </is>
+      </c>
+      <c r="F237" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G237" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H237" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I237" s="3" t="inlineStr">
+        <is>
+          <t>$0.05 a login filled is our estimate; a $3.99 plan is Great at about 8 a day, Costly under about 3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I236"/>
+  <autoFilter ref="A1:I237"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v212: Subscriptions vs Household Services bar moved to Shelf
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$237</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$238</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I237"/>
+  <dimension ref="A1:I238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7991,7 +7991,7 @@
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Moved to Shelf in v212</t>
         </is>
       </c>
       <c r="I166" s="2" t="inlineStr">
@@ -11197,8 +11197,51 @@
         </is>
       </c>
     </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>Subscriptions vs Household Services bar moved from Overview (under the top numbers) to the Shelf tab</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>Overview / Shelf</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H238" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I238" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I237"/>
+  <autoFilter ref="A1:I238"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v213: Domain & Business Registration category (6 registrars, 4 registered agents)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$238</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$239</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I238"/>
+  <dimension ref="A1:I239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11240,8 +11240,55 @@
       </c>
       <c r="I238" s="2" t="inlineStr"/>
     </row>
+    <row r="239">
+      <c r="A239" s="3" t="inlineStr">
+        <is>
+          <t>213</t>
+        </is>
+      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="inlineStr">
+        <is>
+          <t>New category "Domain &amp; Business Registration": 6 domain registrars (Cloudflare, Porkbun, Namecheap, GoDaddy, Squarespace Domains, Hover; yearly .com price) and 4 registered agents (Northwest, ZenBusiness, LegalZoom, Bizee); rated on doing its job and price, with overlap checks for two registrars or two agents</t>
+        </is>
+      </c>
+      <c r="D239" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E239" s="3" t="inlineStr">
+        <is>
+          <t>Explore / Catalog</t>
+        </is>
+      </c>
+      <c r="F239" s="3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G239" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H239" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I239" s="3" t="inlineStr">
+        <is>
+          <t>Prices from comparison sites (etemora.com, Rho, Real Cost Report, Oct 2026), marked unconfirmed; ZenBusiness from its official page. .com renewals may rise slightly around Nov 1, 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I238"/>
+  <autoFilter ref="A1:I239"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v214: Welcome Back on every return, asks before setup, then offers next steps
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$239</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$240</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I239"/>
+  <dimension ref="A1:I240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10961,7 +10961,7 @@
       </c>
       <c r="H232" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v214</t>
         </is>
       </c>
       <c r="I232" s="2" t="inlineStr"/>
@@ -11004,7 +11004,7 @@
       </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v214</t>
         </is>
       </c>
       <c r="I233" s="3" t="inlineStr">
@@ -11287,8 +11287,55 @@
         </is>
       </c>
     </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>214</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>Welcome Back now shows on every return. If details are missing, it lists them and asks "Want to finish setting up now?" (Yes, let's finish / Not now) before any step. When everything is filled in (or after Not now), it says "You're all up to date!" and asks how we can help: Add a subscription, Remove a subscription, Review my subscriptions, Explore cheaper options, or Go to my Overview; a Costly subscription is suggested above the options</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>Welcome Back</t>
+        </is>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G240" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H240" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I240" s="2" t="inlineStr">
+        <is>
+          <t>Once per browser session</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I239"/>
+  <autoFilter ref="A1:I240"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v215: Usage page hides empty sections, moves notes behind i buttons, adds progress bar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$240</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$241</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I240"/>
+  <dimension ref="A1:I241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6742,7 +6742,7 @@
       </c>
       <c r="H139" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v215</t>
         </is>
       </c>
       <c r="I139" s="3" t="inlineStr">
@@ -11334,8 +11334,51 @@
         </is>
       </c>
     </row>
+    <row r="241">
+      <c r="A241" s="3" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="B241" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C241" s="3" t="inlineStr">
+        <is>
+          <t>Usage page simplified for new users: last month's rings, the "not rated" list, the check-in link and the Monthly spending chart (needs 2 months) show only once there is data; page, rings, slider and Real usage explanations moved behind "i" buttons ("How we rate value" fold removed into the page "i"); new "Usage set for X of N" progress bar that fills as sliders are set ("All N set. Nice work!")</t>
+        </is>
+      </c>
+      <c r="D241" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E241" s="3" t="inlineStr">
+        <is>
+          <t>Usage</t>
+        </is>
+      </c>
+      <c r="F241" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G241" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H241" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I241" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I240"/>
+  <autoFilter ref="A1:I241"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v216: Weekly check-in on Usage with an Overview reminder
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$241</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$242</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I241"/>
+  <dimension ref="A1:I242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11377,8 +11377,55 @@
       </c>
       <c r="I241" s="3" t="inlineStr"/>
     </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>216</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>Weekly check-in: "Your weekly check-in is ready" reminder on Overview (Start check-in / Later until tomorrow) and a "How did this week go?" card on Usage (Start / Skip this week). One subscription at a time with its slider where it was, the rating pill follows the slider, Next or "Same as before", "Stop for now"; ends with "All done. Thanks!" and the next check-in date. Due every 7 days once a slider subscription has usage</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>Usage / Overview</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I242" s="2" t="inlineStr">
+        <is>
+          <t>Answers update this month's usage, same as the Usage sliders</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I241"/>
+  <autoFilter ref="A1:I242"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v217: Warehouse clubs rated on money spent, gas and rewards
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$242</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$243</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I242"/>
+  <dimension ref="A1:I243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11424,8 +11424,55 @@
         </is>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" s="3" t="inlineStr">
+        <is>
+          <t>217</t>
+        </is>
+      </c>
+      <c r="B243" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="inlineStr">
+        <is>
+          <t>Warehouse clubs (Costco, Sam's Club) are measured by "Spent there a month, not counting gas" instead of orders, plus an optional "Gallons of gas you buy there a month". Value = 15 cents saved per dollar (+2% back on Executive / Plus) + 20 cents per gallon; Great value when savings are at least 1.2 times the fee, "Saves less than it costs" under 0.9 times. Card shows "Saves you $X a month"</t>
+        </is>
+      </c>
+      <c r="D243" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E243" s="3" t="inlineStr">
+        <is>
+          <t>Usage / Value rating</t>
+        </is>
+      </c>
+      <c r="F243" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G243" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H243" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I243" s="3" t="inlineStr">
+        <is>
+          <t>15% and 20 cents a gallon are our estimates (Consumer Reports 2025 study via IBTimes: Costco ~21% below Walmart; OPIS analyst via CNN 2021); existing real entries are asked again</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I242"/>
+  <autoFilter ref="A1:I243"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v218: Southwest regional providers (AZ, NM)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$243</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$244</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I243"/>
+  <dimension ref="A1:I244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11471,8 +11471,55 @@
         </is>
       </c>
     </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>218</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>Regional providers: Southwest region added (AZ, NM): 18 providers (4 news, 3 internet, 3 fitness, 3 farm shares/co-ops, 2 car wash clubs, 1 home services, 1 pest control, 1 preschool), shown only to users in the states they serve</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>Explore / Regional</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t>8 plan prices from review/comparison sites (not confirmed); many publish no price. regional.json now 192 providers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I243"/>
+  <autoFilter ref="A1:I244"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v219: shared price reports and phone layout fix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$244</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$246</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I244"/>
+  <dimension ref="A1:I246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11518,8 +11518,98 @@
         </is>
       </c>
     </row>
+    <row r="245">
+      <c r="A245" s="3" t="inlineStr">
+        <is>
+          <t>219</t>
+        </is>
+      </c>
+      <c r="B245" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C245" s="3" t="inlineStr">
+        <is>
+          <t>Shared price reports: each price check shows the typical price other members in your area pay (needs 3 reports within 15% of one another) and asks "Is this price right?"; prices you enter are shared without your name. Admin has a Shared price reports table.</t>
+        </is>
+      </c>
+      <c r="D245" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E245" s="3" t="inlineStr">
+        <is>
+          <t>Subscription sheet / Admin</t>
+        </is>
+      </c>
+      <c r="F245" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G245" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H245" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I245" s="3" t="inlineStr">
+        <is>
+          <t>Shared reports work only in the Claude app; the public site has no shared storage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>219</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>Fixed Price check sources showing "[object Object]" and the subscription sheet running wider than the screen on phones.</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>Subscription sheet</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I246" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I244"/>
+  <autoFilter ref="A1:I246"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v220: category breakdown page from Spending by category
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$246</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$247</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I246"/>
+  <dimension ref="A1:I247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11608,8 +11608,55 @@
       </c>
       <c r="I246" s="2" t="inlineStr"/>
     </row>
+    <row r="247">
+      <c r="A247" s="3" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="B247" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C247" s="3" t="inlineStr">
+        <is>
+          <t>Spending by category: tapping a category (slice or legend row) opens its own page with monthly and yearly total, share of total spend, a donut of its subscriptions, each subscription's rating, costly ones called out, and a link to Explore that category.</t>
+        </is>
+      </c>
+      <c r="D247" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E247" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F247" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G247" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H247" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I247" s="3" t="inlineStr">
+        <is>
+          <t>Categories folded into "Other" list every subscription inside them; more than 8 subscriptions fold into a gray slice.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I246"/>
+  <autoFilter ref="A1:I247"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v221: DashPass savings-per-order estimate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$247</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$248</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I247"/>
+  <dimension ref="A1:I248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11655,8 +11655,55 @@
         </is>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>221</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>DoorDash DashPass now has a savings estimate of $4.50 per order (no delivery fee, lower service fee), so it is rated on savings (Great value at 3+ orders a month on $9.99, Costly at 2 or fewer) and shows in What you use most / least.</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>Usage / Subscription sheet</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I248" s="2" t="inlineStr">
+        <is>
+          <t>Estimate from DoorDash's stated $4-$5 average savings per eligible order (ShopBack Oct 2026, RideSharingDriver Jun 2026); users can change it.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I247"/>
+  <autoFilter ref="A1:I248"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v222: usage and price vs typical, value map, admin value rule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$248</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$251</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I248"/>
+  <dimension ref="A1:I251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5145,7 +5145,7 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v222</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr"/>
@@ -11702,8 +11702,149 @@
         </is>
       </c>
     </row>
+    <row r="249">
+      <c r="A249" s="3" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="B249" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C249" s="3" t="inlineStr">
+        <is>
+          <t>Overview: "What you use most / least" replaced by three charts: Your usage vs typical, Your price vs typical, and a Value map (usage across, price up and down, with Keep / Find a cheaper plan / Watch it / Cut or switch corners). Tapping a bar or dot opens the subscription.</t>
+        </is>
+      </c>
+      <c r="D249" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E249" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F249" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G249" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H249" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I249" s="3" t="inlineStr">
+        <is>
+          <t>Long lists show both ends with Show all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>New value rule: where usage and price can both be compared with typical, Great value = usage no more than 10% below typical and price no more than 10% above; Costly = usage 50%+ below or price 25%+ above; Fair otherwise. Admin tab can change the four percentages for everyone.</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>Ratings / Admin</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I250" s="2" t="inlineStr">
+        <is>
+          <t>Older per-category rules still rate anything without a typical figure. Public site: Admin changes last until reload (no shared storage).</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="3" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="B251" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="inlineStr">
+        <is>
+          <t>Typical usage from published averages (video 1.4 h/day Nielsen 2025; music 20.7 h/wk IFPI 2023; AI 3.7 prompts/day OpenAI-NBER 2025; gym 102 visits/yr IHRSA 2010; gaming 8.9 h/wk Video Games Europe 2025; audiobooks 3.8/yr APA 2026; food delivery 3 orders/mo our estimate), replaced by the members' median once 3+ share their usage (no names). Typical price = middle of the closest-priced plan in each catalog service of the same kind.</t>
+        </is>
+      </c>
+      <c r="D251" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E251" s="3" t="inlineStr">
+        <is>
+          <t>Ratings</t>
+        </is>
+      </c>
+      <c r="F251" s="3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G251" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H251" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I251" s="3" t="inlineStr">
+        <is>
+          <t>Music figure covers all listening, so single-app use looks low; audiobook figure covers all listeners, so subscribers look high.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I248"/>
+  <autoFilter ref="A1:I251"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v223: usage measures for protection and always-on services
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$251</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$252</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I251"/>
+  <dimension ref="A1:I252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11843,8 +11843,55 @@
         </is>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>Usage for protection and always-on services (subscription sheet "How much you use it"): car and home insurance = claims in the last 12 months; identity protection and antivirus = alerts reported; security monitoring = alerts plus camera/app checks a week; registered agents = mail forwarded; domains = in use or not. They show on the usage chart and Value map (squares). Low use never says cancel: insurance suggests a better plan or a higher deductible. A domain marked not in use is rated Costly (let it expire or sell it).</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>Subscription sheet / Overview</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H252" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I252" s="2" t="inlineStr">
+        <is>
+          <t>Typical claims from ISO via Insurance Information Institute (car 2024: 11.4 claims per 100 car-years, our sum of coverages; home 2019-2023: 5.6 per 100 homes). Alerts, checks and mail compare with members once 3+ share. Ratings of these services still come from the quote and doing-its-job rules.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I251"/>
+  <autoFilter ref="A1:I252"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v224: welcome inputs match age group tile text
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$252</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$253</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I252"/>
+  <dimension ref="A1:I253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11890,8 +11890,55 @@
         </is>
       </c>
     </row>
+    <row r="253">
+      <c r="A253" s="3" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
+      <c r="B253" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>Welcome pages: every input field (name, country, state, email, search, prices) uses the same text as the age group tiles: bold 22px (19px on small phones) in the accent blue.</t>
+        </is>
+      </c>
+      <c r="D253" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E253" s="3" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F253" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G253" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H253" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I253" s="3" t="inlineStr">
+        <is>
+          <t>Placeholders stay lighter so typed text stands out.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I252"/>
+  <autoFilter ref="A1:I253"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v225: chart descriptions behind info buttons
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$253</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$254</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I253"/>
+  <dimension ref="A1:I254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11937,8 +11937,51 @@
         </is>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>Overview: the descriptions under Your usage vs typical, Your price vs typical and the Value map moved behind an "i" button on each chart.</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I254" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I253"/>
+  <autoFilter ref="A1:I254"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v226: value map usage axis to +500% so heavy use still moves
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$254</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$255</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I254"/>
+  <dimension ref="A1:I255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11980,8 +11980,55 @@
       </c>
       <c r="I254" s="2" t="inlineStr"/>
     </row>
+    <row r="255">
+      <c r="A255" s="3" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="B255" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C255" s="3" t="inlineStr">
+        <is>
+          <t>Value map: usage axis now runs from -100% to +500% of typical (high end squeezed so each doubling gets the same room) instead of stopping at +100%, so heavy use like DoorDash at 8 orders a month (+167%) still moves the dot. The price axis stretches up to +/-200% to fit.</t>
+        </is>
+      </c>
+      <c r="D255" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E255" s="3" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F255" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G255" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H255" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I255" s="3" t="inlineStr">
+        <is>
+          <t>Cuong saw DoorDash not move after changing its orders: anything above +100% was pinned to the edge.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I254"/>
+  <autoFilter ref="A1:I255"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v227: value map axis titles
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$255</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$256</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I255"/>
+  <dimension ref="A1:I256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12027,8 +12027,51 @@
         </is>
       </c>
     </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>Value map: named axes, "Usage vs typical" along the bottom and "Price vs typical" up the left side.</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I256" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I255"/>
+  <autoFilter ref="A1:I256"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v228: Next renewal date in subscription details
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$256</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$257</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I256"/>
+  <dimension ref="A1:I257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12070,8 +12070,51 @@
       </c>
       <c r="I256" s="2" t="inlineStr"/>
     </row>
+    <row r="257">
+      <c r="A257" s="3" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+      <c r="B257" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C257" s="3" t="inlineStr">
+        <is>
+          <t>Added a "Next renewal" date to each subscription's details so you can change when it renews; later renewals follow the billing cycle from that date. Insurance and contract services keep their own "Policy renews" / "Contract or promo renews" date.</t>
+        </is>
+      </c>
+      <c r="D257" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E257" s="3" t="inlineStr">
+        <is>
+          <t>Subscription details</t>
+        </is>
+      </c>
+      <c r="F257" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G257" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H257" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I257" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I256"/>
+  <autoFilter ref="A1:I257"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v229: Costco gas and Kirkland Signature features
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$257</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$258</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I257"/>
+  <dimension ref="A1:I258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12113,8 +12113,55 @@
       </c>
       <c r="I257" s="3" t="inlineStr"/>
     </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>Costco: added "Cheaper gas at Costco gas stations" and "Kirkland Signature products" to Features that matter to me (every membership level).</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>Subscription details</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I258" s="2" t="inlineStr">
+        <is>
+          <t>Gas savings are already counted in Costco's rating as an estimate of about 20 cents a gallon (OPIS via CNN, 2021).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I257"/>
+  <autoFilter ref="A1:I258"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v230: Car insurance compared with drivers like you, yearly quote check
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$258</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$259</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I258"/>
+  <dimension ref="A1:I259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12160,8 +12160,55 @@
         </is>
       </c>
     </row>
+    <row r="259">
+      <c r="A259" s="3" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="B259" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="inlineStr">
+        <is>
+          <t>Car insurance value: compares your price per car with drivers like you (state, main driver's age, coverage, driving record), adds a yearly quote check, and counts a same-coverage quote 15% or more lower as overpaying. Service rating unchanged; claims stay context only.</t>
+        </is>
+      </c>
+      <c r="D259" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E259" s="3" t="inlineStr">
+        <is>
+          <t>Subscription details / Overview</t>
+        </is>
+      </c>
+      <c r="F259" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G259" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H259" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I259" s="3" t="inlineStr">
+        <is>
+          <t>Typical prices are estimates from Insurify's Oct 2026 state averages with age and record factors, replaced by MoSuBi member medians once 3+ similar drivers share.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I258"/>
+  <autoFilter ref="A1:I259"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v231: Inbox in the profile menu with a red badge for new alerts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$259</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$260</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I259"/>
+  <dimension ref="A1:I260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11415,7 +11415,7 @@
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v231</t>
         </is>
       </c>
       <c r="I242" s="2" t="inlineStr">
@@ -12207,8 +12207,51 @@
         </is>
       </c>
     </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>New Inbox in the profile menu. The weekly check-in and "Add your usage" reminders moved there from Overview, along with trial or promo endings and yearly or policy renewals in the next 14 days. A red badge on the profile button counts new items.</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>Profile menu / Overview</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H260" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I260" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I259"/>
+  <autoFilter ref="A1:I260"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v232: Inbox badge no longer clipped on example household pictures
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$260</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$261</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I260"/>
+  <dimension ref="A1:I261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12250,8 +12250,51 @@
       </c>
       <c r="I260" s="2" t="inlineStr"/>
     </row>
+    <row r="261">
+      <c r="A261" s="3" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
+      </c>
+      <c r="B261" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>Inbox badge now sits on top of the profile picture when viewing as an example household (it was clipped inside the circle).</t>
+        </is>
+      </c>
+      <c r="D261" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E261" s="3" t="inlineStr">
+        <is>
+          <t>Header</t>
+        </is>
+      </c>
+      <c r="F261" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G261" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H261" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I261" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I260"/>
+  <autoFilter ref="A1:I261"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v233: Real usage moved to the bottom of Usage and subscription details
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$261</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$262</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I261"/>
+  <dimension ref="A1:I262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12293,8 +12293,51 @@
       </c>
       <c r="I261" s="3" t="inlineStr"/>
     </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>Real usage (use your service's own history) moved to the bottom of the Usage page and of each subscription's details, since it's for advanced users.</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>Usage / Subscription details</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I262" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I261"/>
+  <autoFilter ref="A1:I262"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v234: Insurance details split into sections; car insurance takes every driver
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$262</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$263</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I262"/>
+  <dimension ref="A1:I263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12336,8 +12336,55 @@
       </c>
       <c r="I262" s="2" t="inlineStr"/>
     </row>
+    <row r="263">
+      <c r="A263" s="3" t="inlineStr">
+        <is>
+          <t>234</t>
+        </is>
+      </c>
+      <c r="B263" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>Car and home insurance details: claims rating and your experience moved to a new "Claims and service" section, and the renewal date to "Policy and renewal"; "How it compares" keeps price only. Car insurance now takes every driver on the policy (age and record for each, add or remove drivers).</t>
+        </is>
+      </c>
+      <c r="D263" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E263" s="3" t="inlineStr">
+        <is>
+          <t>Subscription details</t>
+        </is>
+      </c>
+      <c r="F263" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G263" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H263" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I263" s="3" t="inlineStr">
+        <is>
+          <t>Typical price per car averages the drivers' age and record adjustments (our estimate).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I262"/>
+  <autoFilter ref="A1:I263"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v235: Reorder subscription detail sections; usage by month on request
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$263</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$264</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I263"/>
+  <dimension ref="A1:I264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12383,8 +12383,55 @@
         </is>
       </c>
     </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>Subscription details sections reordered: Usage vs cost, Plan and price, How you use it / How it compares, How much you use it, Features that matter to me, Claims and service, Next renewal / Policy and renewal, Alternatives, How hard to switch, Ways to pay less, Real usage. Usage by month is hidden until you tap "Need to correct a past month?" under Usage vs cost.</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr">
+        <is>
+          <t>Subscription details</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G264" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I264" s="2" t="inlineStr">
+        <is>
+          <t>Ask for a lower rate (only when a price is going up) sits right after Plan and price.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I263"/>
+  <autoFilter ref="A1:I264"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v236: Pacific regional providers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$264</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$265</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I264"/>
+  <dimension ref="A1:I265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12430,8 +12430,55 @@
         </is>
       </c>
     </row>
+    <row r="265">
+      <c r="A265" s="3" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="B265" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="inlineStr">
+        <is>
+          <t>Added 23 Pacific regional providers (CA, OR, WA, AK, HI): internet, mobile, news, fitness, food, car wash, green power and pest control. They show only to people in the states they serve. 215 regional providers in all.</t>
+        </is>
+      </c>
+      <c r="D265" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E265" s="3" t="inlineStr">
+        <is>
+          <t>Explore / Regional</t>
+        </is>
+      </c>
+      <c r="F265" s="3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G265" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H265" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I265" s="3" t="inlineStr">
+        <is>
+          <t>10 have a missing or unconfirmed price; see regional/pacific-report.md.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I264"/>
+  <autoFilter ref="A1:I265"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v237: Connected car, driver assist and satellite radio subscriptions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$265</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$266</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I265"/>
+  <dimension ref="A1:I266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12477,8 +12477,55 @@
         </is>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>237</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>New Explore categories for carmaker subscriptions: Connected Car (18: car alerts, remote start, phone as key, Wi-Fi), Driver Assist &amp; Self-Driving (6: Tesla FSD, Super Cruise, BlueCruise, BMW, Mercedes, ProPILOT) and Satellite Radio (SiriusXM). Usage measured in days used a month (listening hours for SiriusXM).</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr">
+        <is>
+          <t>Explore / Catalog</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G266" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H266" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I266" s="2" t="inlineStr">
+        <is>
+          <t>Prices from official pages where possible; BMW, Mercedes, Lexus, Genesis, Honda, Acura, Nissan and some Subaru, Volvo and Hyundai prices come from news or review sites and are marked as estimates.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I265"/>
+  <autoFilter ref="A1:I266"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v238: Sports streaming, sports ticket passes and theme park passes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$266</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$267</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I266"/>
+  <dimension ref="A1:I267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12524,8 +12524,55 @@
         </is>
       </c>
     </row>
+    <row r="267">
+      <c r="A267" s="3" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="B267" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="inlineStr">
+        <is>
+          <t>New Explore categories: Sports Streaming (11: NFL Sunday Ticket, NFL+, NBA League Pass, MLB.TV, ESPN, NHL Power Play, WNBA, DAZN, Tennis Channel, B1G+, FloSports), Sports Ticket Passes (22 team passes: 17 MLB ballpark passes, 2 NHL, 3 college; shown only in the team's state) and Theme Park Passes (17: Disney, Universal, Six Flags, SeaWorld, Busch Gardens, Legoland, Dollywood, Hersheypark and more; shown only where the parks are).</t>
+        </is>
+      </c>
+      <c r="D267" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E267" s="3" t="inlineStr">
+        <is>
+          <t>Explore / Catalog</t>
+        </is>
+      </c>
+      <c r="F267" s="3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G267" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H267" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I267" s="3" t="inlineStr">
+        <is>
+          <t>Many prices are sales or change by park; unconfirmed ones (from news or review sites) are labeled estimates. No current passes found for most MLB teams, any NBA, MLS or WNBA team.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I266"/>
+  <autoFilter ref="A1:I267"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v239: New welcome description
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$267</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$268</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I267"/>
+  <dimension ref="A1:I268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12571,8 +12571,51 @@
         </is>
       </c>
     </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>239</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>Welcome page description replaced with Cuong's new two-paragraph text ("The average American spends about $1,080 a year on subscriptions and recurring services..." / "At MoSuBi, we use AI, market research, and information you share...").</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E268" s="2" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F268" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G268" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H268" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I268" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I267"/>
+  <autoFilter ref="A1:I268"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v240: Welcome step heading reads Let's get started
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$268</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$269</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I268"/>
+  <dimension ref="A1:I269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12614,8 +12614,51 @@
       </c>
       <c r="I268" s="2" t="inlineStr"/>
     </row>
+    <row r="269">
+      <c r="A269" s="3" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="B269" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C269" s="3" t="inlineStr">
+        <is>
+          <t>Second welcome page heading changed from "We're Glad You're Here!" to "Let's get started."</t>
+        </is>
+      </c>
+      <c r="D269" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E269" s="3" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F269" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G269" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H269" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I269" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I268"/>
+  <autoFilter ref="A1:I269"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v241: Shorter second welcome paragraph
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$269</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$270</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I269"/>
+  <dimension ref="A1:I270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12609,7 +12609,7 @@
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v241</t>
         </is>
       </c>
       <c r="I268" s="2" t="inlineStr"/>
@@ -12657,8 +12657,51 @@
       </c>
       <c r="I269" s="3" t="inlineStr"/>
     </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>241</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>Welcome page second paragraph now reads "At MoSuBi, we use AI and market research to help you get the most for your money."</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G270" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H270" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I270" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I269"/>
+  <autoFilter ref="A1:I270"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v242: New second welcome page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$270</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$271</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I270"/>
+  <dimension ref="A1:I271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12652,7 +12652,7 @@
       </c>
       <c r="H269" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Removed in v242</t>
         </is>
       </c>
       <c r="I269" s="3" t="inlineStr"/>
@@ -12700,8 +12700,51 @@
       </c>
       <c r="I270" s="2" t="inlineStr"/>
     </row>
+    <row r="271">
+      <c r="A271" s="3" t="inlineStr">
+        <is>
+          <t>242</t>
+        </is>
+      </c>
+      <c r="B271" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C271" s="3" t="inlineStr">
+        <is>
+          <t>New second welcome page: "No gimmick, no fluff. We're here to help so let's get started!" in gold, centered, with Back and Next. The "Let's get started." heading on the About you page (now the third page) was removed.</t>
+        </is>
+      </c>
+      <c r="D271" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E271" s="3" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F271" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G271" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H271" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I271" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I270"/>
+  <autoFilter ref="A1:I271"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v243: Welcome pages line up; MoSuBi in logo green
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$271</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$272</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I271"/>
+  <dimension ref="A1:I272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12738,13 +12738,56 @@
       </c>
       <c r="H271" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v243</t>
         </is>
       </c>
       <c r="I271" s="3" t="inlineStr"/>
     </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>243</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>Welcome pages: "MoSuBi" in the first page's text is logo green (#4ade80). The second page now opens with a gold "Let's get started!" where the first page's title sits, then "No gimmick, no fluff. We're here to help.", with Back and Next lined up with the first page's Next button.</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G272" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H272" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I272" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I271"/>
+  <autoFilter ref="A1:I272"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v244: welcome pages 3-4 section headers match pages 1-2 text size
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$272</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$273</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I272"/>
+  <dimension ref="A1:I273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12786,8 +12786,51 @@
       </c>
       <c r="I272" s="2" t="inlineStr"/>
     </row>
+    <row r="273">
+      <c r="A273" s="3" t="inlineStr">
+        <is>
+          <t>244</t>
+        </is>
+      </c>
+      <c r="B273" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C273" s="3" t="inlineStr">
+        <is>
+          <t>Welcome pages 3 and 4: the numbered section headers (Tell us about yourself, My age group, Which subscriptions, Browse by category and the rest) now use the same size as the text on pages 1 and 2 (21px, 20px on phones) in the main text color (white in dark mode)</t>
+        </is>
+      </c>
+      <c r="D273" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E273" s="3" t="inlineStr">
+        <is>
+          <t>Welcome</t>
+        </is>
+      </c>
+      <c r="F273" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G273" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H273" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I273" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I272"/>
+  <autoFilter ref="A1:I273"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v245: MoSuBi header name in logo green on all pages
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$273</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$274</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I273"/>
+  <dimension ref="A1:I274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12829,8 +12829,51 @@
       </c>
       <c r="I273" s="3" t="inlineStr"/>
     </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>245</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>The MoSuBi name in the header is now logo green (#4ade80) on every page after the welcome pages, matching the welcome pages</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E274" s="2" t="inlineStr">
+        <is>
+          <t>All pages (header)</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G274" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H274" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I274" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I273"/>
+  <autoFilter ref="A1:I274"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v246: Sports Ticket Passes browse by league, then team
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$274</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$275</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I274"/>
+  <dimension ref="A1:I275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12872,8 +12872,55 @@
       </c>
       <c r="I274" s="2" t="inlineStr"/>
     </row>
+    <row r="275">
+      <c r="A275" s="3" t="inlineStr">
+        <is>
+          <t>246</t>
+        </is>
+      </c>
+      <c r="B275" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C275" s="3" t="inlineStr">
+        <is>
+          <t>Sports Ticket Passes are browsed league first: tiles for MLB, NHL and College (our own text badges, not league logos, which are trademarks). Tapping a league opens its page with teams near you first, then every other team with a pass. Works on the welcome picker, Add subscriptions and Explore; out-of-state teams can now be picked and searched</t>
+        </is>
+      </c>
+      <c r="D275" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E275" s="3" t="inlineStr">
+        <is>
+          <t>Welcome / Explore</t>
+        </is>
+      </c>
+      <c r="F275" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G275" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H275" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I275" s="3" t="inlineStr">
+        <is>
+          <t>Each pass in explore-extra.json now has a league field (MLB 17, NHL 2, College 3). No NFL or NBA passes found yet.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I274"/>
+  <autoFilter ref="A1:I275"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v247: medium gray card border for more contrast
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$275</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$276</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I275"/>
+  <dimension ref="A1:I276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10570,7 +10570,7 @@
       </c>
       <c r="H223" s="3" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Changed in v247</t>
         </is>
       </c>
       <c r="I223" s="3" t="inlineStr">
@@ -12919,8 +12919,55 @@
         </is>
       </c>
     </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>247</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>Widget cards get a stronger medium gray border for more contrast (#a3b1c6 light, #44547a dark), option B of three mocked up</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>All pages</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H276" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I276" s="2" t="inlineStr">
+        <is>
+          <t>Mockups in design/contrast/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I275"/>
+  <autoFilter ref="A1:I276"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v248: remove extra gap below Spending by category
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$276</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$277</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I276"/>
+  <dimension ref="A1:I277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12966,8 +12966,51 @@
         </is>
       </c>
     </row>
+    <row r="277">
+      <c r="A277" s="3" t="inlineStr">
+        <is>
+          <t>248</t>
+        </is>
+      </c>
+      <c r="B277" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C277" s="3" t="inlineStr">
+        <is>
+          <t>Overview: removed the extra space below Spending by category (34px gap down to 14px, like the other cards). Cards inside a chart grid no longer add their own 20px bottom margin</t>
+        </is>
+      </c>
+      <c r="D277" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E277" s="3" t="inlineStr">
+        <is>
+          <t>Overview / Usage</t>
+        </is>
+      </c>
+      <c r="F277" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="G277" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H277" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I277" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I276"/>
+  <autoFilter ref="A1:I277"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v249: Welcome Back Help Center; help question moved and enlarged
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$277</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$279</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I277"/>
+  <dimension ref="A1:I279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13009,8 +13009,98 @@
       </c>
       <c r="I277" s="3" t="inlineStr"/>
     </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>249</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>Welcome Back: new Help Center with four guides (Surprise price increase, Payment dispute, Find contact info, Plan changes). Each opens step-by-step help plus your subscriptions: tap one to update its price or plan, or open its official site and a help search</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr">
+        <is>
+          <t>Welcome Back</t>
+        </is>
+      </c>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="G278" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H278" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I278" s="2" t="inlineStr">
+        <is>
+          <t>General guidance. No phone numbers listed yet; contact info links to the official site and a web search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="3" t="inlineStr">
+        <is>
+          <t>249</t>
+        </is>
+      </c>
+      <c r="B279" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>Welcome Back: "Is there anything we can help you with today?" moved below the Costly subscription card and enlarged to the welcome section header size (21px, 20px on phones)</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E279" s="3" t="inlineStr">
+        <is>
+          <t>Welcome Back</t>
+        </is>
+      </c>
+      <c r="F279" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G279" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H279" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I279" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I277"/>
+  <autoFilter ref="A1:I279"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v250: official support contacts for 23 popular services in Help Center
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$279</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$280</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I279"/>
+  <dimension ref="A1:I280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13099,8 +13099,55 @@
       </c>
       <c r="I279" s="3" t="inlineStr"/>
     </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>Help Center &gt; Find contact info now shows the official way to reach support for 23 popular services (how to contact, official contact page, phone number only where the service publishes one), listed first. Other services keep the official site and help search links</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E280" s="2" t="inlineStr">
+        <is>
+          <t>Welcome Back</t>
+        </is>
+      </c>
+      <c r="F280" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G280" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H280" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I280" s="2" t="inlineStr">
+        <is>
+          <t>contacts.json, taken only from each service's own help pages (scam numbers dominate search results). Only Apple publishes a phone number (1-800-275-2273). Hulu and NYT not yet confirmed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I279"/>
+  <autoFilter ref="A1:I280"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v251: Selection Summary heading after the welcome flow
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwR3W7uoJz7e2kL7uW3DcJ
</commit_message>
<xml_diff>
--- a/changelog/change-log.xlsx
+++ b/changelog/change-log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$280</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Log'!$A$1:$I$281</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I280"/>
+  <dimension ref="A1:I281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13146,8 +13146,51 @@
         </is>
       </c>
     </row>
+    <row r="281">
+      <c r="A281" s="3" t="inlineStr">
+        <is>
+          <t>251</t>
+        </is>
+      </c>
+      <c r="B281" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C281" s="3" t="inlineStr">
+        <is>
+          <t>When the welcome flow ends (Done after setting up, or Next with nothing new to set up), the Overview heading reads "Selection Summary" instead of the greeting. Leaving Overview brings the greeting back</t>
+        </is>
+      </c>
+      <c r="D281" s="3" t="inlineStr">
+        <is>
+          <t>Cuong</t>
+        </is>
+      </c>
+      <c r="E281" s="3" t="inlineStr">
+        <is>
+          <t>Overview / Welcome</t>
+        </is>
+      </c>
+      <c r="F281" s="3" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G281" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H281" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I281" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I280"/>
+  <autoFilter ref="A1:I281"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>